<commit_message>
GLB - Milly Update
</commit_message>
<xml_diff>
--- a/Sinner_Stuff/dispatch.xlsx
+++ b/Sinner_Stuff/dispatch.xlsx
@@ -28499,86 +28499,86 @@
     </row>
     <row r="181">
       <c r="A181" t="n">
-        <v>1099001</v>
+        <v>1056001</v>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>Green</t>
+          <t>Purple</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>Dream Interpretation</t>
+          <t>Cupid's Arrow</t>
         </is>
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>夢の解析</t>
+          <t>キューピットの矢</t>
         </is>
       </c>
       <c r="E181" t="inlineStr">
         <is>
-          <t>꿈의 해석</t>
+          <t>큐피트의 화살</t>
         </is>
       </c>
       <c r="F181" t="inlineStr">
         <is>
-          <t>梦的解析</t>
+          <t>丘比特之箭</t>
         </is>
       </c>
       <c r="G181" t="inlineStr">
         <is>
-          <t>夢的解析</t>
+          <t>丘比特之箭</t>
         </is>
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>Residents in some areas of Eastside often suffer from nightmares. It is necessary to find out why.</t>
+          <t>A dating show in Eastside is recruiting volunteers. Several Sinners, intrigued by the opportunity, eagerly request to join.</t>
         </is>
       </c>
       <c r="I181" t="inlineStr">
         <is>
-          <t>ニューシティの一部エリアの住民がよくナイトメアにうなされている。具体的な原因を調査しなければならない。</t>
+          <t>ニューシティで行われる婚活イベントのボランティアスタッフの募集が始まったと聞き、やる気を見せているコンビクトがいる。</t>
         </is>
       </c>
       <c r="J181" t="inlineStr">
         <is>
-          <t>신성 일부 지역 주민들은 악몽을 자주꾼다. 구체적인 원인을 철저히 조사해야 한다.</t>
+          <t>신성의 어느 연애 프로그램에서 지원자를 모집하고 있다. 일부 수감자들이 소식을 듣고 적극적으로 참여하려 한다.</t>
         </is>
       </c>
       <c r="K181" t="inlineStr">
         <is>
-          <t>新城一些区域的居民经常做噩梦，需要查清具体原因。</t>
+          <t>新城某相亲节目正在招募志愿者， 有禁闭者听说后积极要求参加。</t>
         </is>
       </c>
       <c r="L181" t="inlineStr">
         <is>
-          <t>新城一些區域的居民經常做惡夢，需要查明具體原因。</t>
+          <t>新城某相親節目正在招募志工， 有禁閉者聽說後積極要求參加。</t>
         </is>
       </c>
       <c r="M181" t="inlineStr">
         <is>
-          <t>Hecate</t>
+          <t>Milly</t>
         </is>
       </c>
       <c r="N181" t="inlineStr">
         <is>
-          <t>ヘカテー</t>
+          <t>ミリー</t>
         </is>
       </c>
       <c r="O181" t="inlineStr">
         <is>
-          <t>헤카테</t>
+          <t>밀리</t>
         </is>
       </c>
       <c r="P181" t="inlineStr">
         <is>
-          <t>赫卡蒂</t>
+          <t>蜜莉</t>
         </is>
       </c>
       <c r="Q181" t="inlineStr">
         <is>
-          <t>赫卡蒂</t>
+          <t>蜜莉</t>
         </is>
       </c>
       <c r="R181" t="inlineStr"/>
@@ -28588,60 +28588,1000 @@
       <c r="V181" t="inlineStr"/>
       <c r="W181" t="inlineStr">
         <is>
+          <t>Hypercube</t>
+        </is>
+      </c>
+      <c r="X181" t="inlineStr">
+        <is>
+          <t>イレギュラーキューブ</t>
+        </is>
+      </c>
+      <c r="Y181" t="inlineStr">
+        <is>
+          <t>큐브</t>
+        </is>
+      </c>
+      <c r="Z181" t="inlineStr">
+        <is>
+          <t>异方晶</t>
+        </is>
+      </c>
+      <c r="AA181" t="inlineStr">
+        <is>
+          <t>異方晶</t>
+        </is>
+      </c>
+      <c r="AB181" t="inlineStr">
+        <is>
+          <t>30.0</t>
+        </is>
+      </c>
+      <c r="AC181" t="inlineStr">
+        <is>
+          <t>Hypercube</t>
+        </is>
+      </c>
+      <c r="AD181" t="inlineStr">
+        <is>
+          <t>イレギュラーキューブ</t>
+        </is>
+      </c>
+      <c r="AE181" t="inlineStr">
+        <is>
+          <t>큐브</t>
+        </is>
+      </c>
+      <c r="AF181" t="inlineStr">
+        <is>
+          <t>异方晶</t>
+        </is>
+      </c>
+      <c r="AG181" t="inlineStr">
+        <is>
+          <t>異方晶</t>
+        </is>
+      </c>
+      <c r="AH181" t="inlineStr">
+        <is>
+          <t>10.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="n">
+        <v>1056002</v>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>Green</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>Wine Tasting</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>試飲会</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>주류 시음회</t>
+        </is>
+      </c>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>品酒会</t>
+        </is>
+      </c>
+      <c r="G182" t="inlineStr">
+        <is>
+          <t>品酒會</t>
+        </is>
+      </c>
+      <c r="H182" t="inlineStr">
+        <is>
+          <t>The Bureau is sourcing new alcoholic beverages and has organized a tasting event, inviting experienced Sinners to participate and provide their opinions.</t>
+        </is>
+      </c>
+      <c r="I182" t="inlineStr">
+        <is>
+          <t>お酒の仕入れを行うため、管理局で試飲会を開くことに。そこで、その方面に詳しいコンビクトがアドバイザーとして呼ばれた。</t>
+        </is>
+      </c>
+      <c r="J182" t="inlineStr">
+        <is>
+          <t>관리국에서 주류를 구매하려 한다. 경험이 있는 수감자를 초청하여 조언을 구하는 시음회를 주최할 예정이다.</t>
+        </is>
+      </c>
+      <c r="K182" t="inlineStr">
+        <is>
+          <t>管理局计划采购酒水，因此组织了一场试喝会，邀请有经验的禁闭者参加并提供建议。</t>
+        </is>
+      </c>
+      <c r="L182" t="inlineStr">
+        <is>
+          <t>管理局計畫採購酒水，因此組織了一場試喝會，邀請有經驗的禁閉者參加並提供建議。</t>
+        </is>
+      </c>
+      <c r="M182" t="inlineStr">
+        <is>
+          <t>Cassian</t>
+        </is>
+      </c>
+      <c r="N182" t="inlineStr">
+        <is>
+          <t>キャシアン</t>
+        </is>
+      </c>
+      <c r="O182" t="inlineStr">
+        <is>
+          <t>카시안</t>
+        </is>
+      </c>
+      <c r="P182" t="inlineStr">
+        <is>
+          <t>卡兹安</t>
+        </is>
+      </c>
+      <c r="Q182" t="inlineStr">
+        <is>
+          <t>卡茲安</t>
+        </is>
+      </c>
+      <c r="R182" t="inlineStr"/>
+      <c r="S182" t="inlineStr"/>
+      <c r="T182" t="inlineStr"/>
+      <c r="U182" t="inlineStr"/>
+      <c r="V182" t="inlineStr"/>
+      <c r="W182" t="inlineStr">
+        <is>
+          <t>Hypercube</t>
+        </is>
+      </c>
+      <c r="X182" t="inlineStr">
+        <is>
+          <t>イレギュラーキューブ</t>
+        </is>
+      </c>
+      <c r="Y182" t="inlineStr">
+        <is>
+          <t>큐브</t>
+        </is>
+      </c>
+      <c r="Z182" t="inlineStr">
+        <is>
+          <t>异方晶</t>
+        </is>
+      </c>
+      <c r="AA182" t="inlineStr">
+        <is>
+          <t>異方晶</t>
+        </is>
+      </c>
+      <c r="AB182" t="inlineStr">
+        <is>
+          <t>10.0</t>
+        </is>
+      </c>
+      <c r="AC182" t="inlineStr">
+        <is>
+          <t>Hypercube</t>
+        </is>
+      </c>
+      <c r="AD182" t="inlineStr">
+        <is>
+          <t>イレギュラーキューブ</t>
+        </is>
+      </c>
+      <c r="AE182" t="inlineStr">
+        <is>
+          <t>큐브</t>
+        </is>
+      </c>
+      <c r="AF182" t="inlineStr">
+        <is>
+          <t>异方晶</t>
+        </is>
+      </c>
+      <c r="AG182" t="inlineStr">
+        <is>
+          <t>異方晶</t>
+        </is>
+      </c>
+      <c r="AH182" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="n">
+        <v>1056003</v>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>Blue</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>Music Appreciation</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>音楽鑑賞</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>음악 감상</t>
+        </is>
+      </c>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t>音乐鉴赏</t>
+        </is>
+      </c>
+      <c r="G183" t="inlineStr">
+        <is>
+          <t>音樂鑑賞</t>
+        </is>
+      </c>
+      <c r="H183" t="inlineStr">
+        <is>
+          <t>The Bureau is sending agents undercover to infiltrate a music appreciation gathering in Eastside. To maintain their cover, they require Sinners with a working knowledge of classical music to accompany them.</t>
+        </is>
+      </c>
+      <c r="I183" t="inlineStr">
+        <is>
+          <t>ニューシティで行われる音楽鑑賞会の実情を探るため、管理局から人が送られることとなった。不要な疑いをかけられないためにも、クラシック音楽に詳しいコンビクトの付き添いが必要だ。</t>
+        </is>
+      </c>
+      <c r="J183" t="inlineStr">
+        <is>
+          <t>관리국에서 인원을 파견하여 신성의 어느 음악 감상회에 잠입시킬 예정이다. 의심을 받지 않기 위해, 클래식 음악을 아는 수감자들이 동반 입장해야 한다.</t>
+        </is>
+      </c>
+      <c r="K183" t="inlineStr">
+        <is>
+          <t>管理局将派出探员卧底新城某音乐鉴赏会，为避免遭到怀疑，现需几位对古典音乐略通一二的禁闭者陪同入场。</t>
+        </is>
+      </c>
+      <c r="L183" t="inlineStr">
+        <is>
+          <t>管理局將派出探員臥底新城某音樂鑑賞會，為避免遭到懷疑，現需幾位對古典音樂略通一二的禁閉者陪同入場。</t>
+        </is>
+      </c>
+      <c r="M183" t="inlineStr">
+        <is>
+          <t>Cassian</t>
+        </is>
+      </c>
+      <c r="N183" t="inlineStr">
+        <is>
+          <t>キャシアン</t>
+        </is>
+      </c>
+      <c r="O183" t="inlineStr">
+        <is>
+          <t>카시안</t>
+        </is>
+      </c>
+      <c r="P183" t="inlineStr">
+        <is>
+          <t>卡兹安</t>
+        </is>
+      </c>
+      <c r="Q183" t="inlineStr">
+        <is>
+          <t>卡茲安</t>
+        </is>
+      </c>
+      <c r="R183" t="inlineStr">
+        <is>
+          <t>Ariel</t>
+        </is>
+      </c>
+      <c r="S183" t="inlineStr">
+        <is>
+          <t>アリエル</t>
+        </is>
+      </c>
+      <c r="T183" t="inlineStr">
+        <is>
+          <t>아리엘</t>
+        </is>
+      </c>
+      <c r="U183" t="inlineStr">
+        <is>
+          <t>艾瑞尔</t>
+        </is>
+      </c>
+      <c r="V183" t="inlineStr">
+        <is>
+          <t>艾瑞爾</t>
+        </is>
+      </c>
+      <c r="W183" t="inlineStr">
+        <is>
+          <t>Hypercube</t>
+        </is>
+      </c>
+      <c r="X183" t="inlineStr">
+        <is>
+          <t>イレギュラーキューブ</t>
+        </is>
+      </c>
+      <c r="Y183" t="inlineStr">
+        <is>
+          <t>큐브</t>
+        </is>
+      </c>
+      <c r="Z183" t="inlineStr">
+        <is>
+          <t>异方晶</t>
+        </is>
+      </c>
+      <c r="AA183" t="inlineStr">
+        <is>
+          <t>異方晶</t>
+        </is>
+      </c>
+      <c r="AB183" t="inlineStr">
+        <is>
+          <t>15.0</t>
+        </is>
+      </c>
+      <c r="AC183" t="inlineStr">
+        <is>
+          <t>Hypercube</t>
+        </is>
+      </c>
+      <c r="AD183" t="inlineStr">
+        <is>
+          <t>イレギュラーキューブ</t>
+        </is>
+      </c>
+      <c r="AE183" t="inlineStr">
+        <is>
+          <t>큐브</t>
+        </is>
+      </c>
+      <c r="AF183" t="inlineStr">
+        <is>
+          <t>异方晶</t>
+        </is>
+      </c>
+      <c r="AG183" t="inlineStr">
+        <is>
+          <t>異方晶</t>
+        </is>
+      </c>
+      <c r="AH183" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="n">
+        <v>1057001</v>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>Purple</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>Circus Mystery</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>###</t>
+        </is>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>###</t>
+        </is>
+      </c>
+      <c r="F184" t="inlineStr">
+        <is>
+          <t>马戏团疑云</t>
+        </is>
+      </c>
+      <c r="G184" t="inlineStr">
+        <is>
+          <t>馬戲團疑雲</t>
+        </is>
+      </c>
+      <c r="H184" t="inlineStr">
+        <is>
+          <t>A renowned circus in Eastside is currently embroiled in an abuse scandal. The Public Security Bureau urgently requires a physically robust Sinner with a distinctive appearance to infiltrate the troupe undercover and investigate the allegations.</t>
+        </is>
+      </c>
+      <c r="I184" t="inlineStr">
+        <is>
+          <t>###</t>
+        </is>
+      </c>
+      <c r="J184" t="inlineStr">
+        <is>
+          <t>###</t>
+        </is>
+      </c>
+      <c r="K184" t="inlineStr">
+        <is>
+          <t>近期，新城一家知名马戏团深陷虐待丑闻，治安局急需一名实力强劲、外表异于常人的禁闭者前去应聘，潜伏调查。</t>
+        </is>
+      </c>
+      <c r="L184" t="inlineStr">
+        <is>
+          <t>近期，新城一家知名馬戲團深陷虐待醜聞，治安局急需一名實力強勁、外表異於常人的禁閉者前去應聘，潛伏調查。</t>
+        </is>
+      </c>
+      <c r="M184" t="inlineStr">
+        <is>
+          <t>Synex</t>
+        </is>
+      </c>
+      <c r="N184" t="inlineStr">
+        <is>
+          <t>シニックス</t>
+        </is>
+      </c>
+      <c r="O184" t="inlineStr">
+        <is>
+          <t>시넥스</t>
+        </is>
+      </c>
+      <c r="P184" t="inlineStr">
+        <is>
+          <t>西涅克斯</t>
+        </is>
+      </c>
+      <c r="Q184" t="inlineStr">
+        <is>
+          <t>西涅克斯</t>
+        </is>
+      </c>
+      <c r="R184" t="inlineStr"/>
+      <c r="S184" t="inlineStr"/>
+      <c r="T184" t="inlineStr"/>
+      <c r="U184" t="inlineStr"/>
+      <c r="V184" t="inlineStr"/>
+      <c r="W184" t="inlineStr">
+        <is>
+          <t>DisCoins</t>
+        </is>
+      </c>
+      <c r="X184" t="inlineStr">
+        <is>
+          <t>ディスコイン</t>
+        </is>
+      </c>
+      <c r="Y184" t="inlineStr">
+        <is>
+          <t>디스코인</t>
+        </is>
+      </c>
+      <c r="Z184" t="inlineStr">
+        <is>
+          <t>狄斯币</t>
+        </is>
+      </c>
+      <c r="AA184" t="inlineStr">
+        <is>
+          <t>狄斯幣</t>
+        </is>
+      </c>
+      <c r="AB184" t="inlineStr">
+        <is>
+          <t>8000.0</t>
+        </is>
+      </c>
+      <c r="AC184" t="inlineStr">
+        <is>
+          <t>DisCoins</t>
+        </is>
+      </c>
+      <c r="AD184" t="inlineStr">
+        <is>
+          <t>ディスコイン</t>
+        </is>
+      </c>
+      <c r="AE184" t="inlineStr">
+        <is>
+          <t>디스코인</t>
+        </is>
+      </c>
+      <c r="AF184" t="inlineStr">
+        <is>
+          <t>狄斯币</t>
+        </is>
+      </c>
+      <c r="AG184" t="inlineStr">
+        <is>
+          <t>狄斯幣</t>
+        </is>
+      </c>
+      <c r="AH184" t="inlineStr">
+        <is>
+          <t>2000.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="n">
+        <v>1057002</v>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>Green</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>Square Clean-up</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>###</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>###</t>
+        </is>
+      </c>
+      <c r="F185" t="inlineStr">
+        <is>
+          <t>广场清洁</t>
+        </is>
+      </c>
+      <c r="G185" t="inlineStr">
+        <is>
+          <t>廣場清潔</t>
+        </is>
+      </c>
+      <c r="H185" t="inlineStr">
+        <is>
+          <t>With large crowds expected for the festival, the sanitation department is short-staffed for cleaning the main square. They are urgently recruiting Sinners adept at general labor to assist with the workload.</t>
+        </is>
+      </c>
+      <c r="I185" t="inlineStr">
+        <is>
+          <t>###</t>
+        </is>
+      </c>
+      <c r="J185" t="inlineStr">
+        <is>
+          <t>###</t>
+        </is>
+      </c>
+      <c r="K185" t="inlineStr">
+        <is>
+          <t>由于节庆期间的线下人流过大，负责打扫广场的环卫部门人手紧张，现紧急借调擅长杂勤的禁闭者参与作业。</t>
+        </is>
+      </c>
+      <c r="L185" t="inlineStr">
+        <is>
+          <t>由於節慶期間的線下人流過大，負責打掃廣場的環衛部門人手不足，現緊急借調擅長雜勤的禁閉者參與作業。</t>
+        </is>
+      </c>
+      <c r="M185" t="inlineStr">
+        <is>
+          <t>Thani</t>
+        </is>
+      </c>
+      <c r="N185" t="inlineStr">
+        <is>
+          <t>###</t>
+        </is>
+      </c>
+      <c r="O185" t="inlineStr">
+        <is>
+          <t>사니</t>
+        </is>
+      </c>
+      <c r="P185" t="inlineStr">
+        <is>
+          <t>萨妮</t>
+        </is>
+      </c>
+      <c r="Q185" t="inlineStr">
+        <is>
+          <t>薩妮</t>
+        </is>
+      </c>
+      <c r="R185" t="inlineStr"/>
+      <c r="S185" t="inlineStr"/>
+      <c r="T185" t="inlineStr"/>
+      <c r="U185" t="inlineStr"/>
+      <c r="V185" t="inlineStr"/>
+      <c r="W185" t="inlineStr">
+        <is>
+          <t>DisCoins</t>
+        </is>
+      </c>
+      <c r="X185" t="inlineStr">
+        <is>
+          <t>ディスコイン</t>
+        </is>
+      </c>
+      <c r="Y185" t="inlineStr">
+        <is>
+          <t>디스코인</t>
+        </is>
+      </c>
+      <c r="Z185" t="inlineStr">
+        <is>
+          <t>狄斯币</t>
+        </is>
+      </c>
+      <c r="AA185" t="inlineStr">
+        <is>
+          <t>狄斯幣</t>
+        </is>
+      </c>
+      <c r="AB185" t="inlineStr">
+        <is>
+          <t>2400.0</t>
+        </is>
+      </c>
+      <c r="AC185" t="inlineStr">
+        <is>
+          <t>DisCoins</t>
+        </is>
+      </c>
+      <c r="AD185" t="inlineStr">
+        <is>
+          <t>ディスコイン</t>
+        </is>
+      </c>
+      <c r="AE185" t="inlineStr">
+        <is>
+          <t>디스코인</t>
+        </is>
+      </c>
+      <c r="AF185" t="inlineStr">
+        <is>
+          <t>狄斯币</t>
+        </is>
+      </c>
+      <c r="AG185" t="inlineStr">
+        <is>
+          <t>狄斯幣</t>
+        </is>
+      </c>
+      <c r="AH185" t="inlineStr">
+        <is>
+          <t>800.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="n">
+        <v>1057003</v>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>Blue</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>Covert Infiltration</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>###</t>
+        </is>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>###</t>
+        </is>
+      </c>
+      <c r="F186" t="inlineStr">
+        <is>
+          <t>伪装潜入</t>
+        </is>
+      </c>
+      <c r="G186" t="inlineStr">
+        <is>
+          <t>偽裝潛入</t>
+        </is>
+      </c>
+      <c r="H186" t="inlineStr">
+        <is>
+          <t>According to latest reports, a hotel in Eastside has been seized by hostage-takers. They urgently need two Sinners to disguise themselves as service staff, infiltrate the building, and ensure the safety of the hostages.</t>
+        </is>
+      </c>
+      <c r="I186" t="inlineStr">
+        <is>
+          <t>###</t>
+        </is>
+      </c>
+      <c r="J186" t="inlineStr">
+        <is>
+          <t>###</t>
+        </is>
+      </c>
+      <c r="K186" t="inlineStr">
+        <is>
+          <t>据最新消息称，新城某酒店遭到劫持，急需两名禁闭者伪装服务人员混入现场，保护人质安全。</t>
+        </is>
+      </c>
+      <c r="L186" t="inlineStr">
+        <is>
+          <t>據最新消息稱，新城某飯店遭到劫持，急需兩名禁閉者偽裝服務人員混入現場，保護人質安全。</t>
+        </is>
+      </c>
+      <c r="M186" t="inlineStr">
+        <is>
+          <t>Thani</t>
+        </is>
+      </c>
+      <c r="N186" t="inlineStr">
+        <is>
+          <t>###</t>
+        </is>
+      </c>
+      <c r="O186" t="inlineStr">
+        <is>
+          <t>사니</t>
+        </is>
+      </c>
+      <c r="P186" t="inlineStr">
+        <is>
+          <t>萨妮</t>
+        </is>
+      </c>
+      <c r="Q186" t="inlineStr">
+        <is>
+          <t>薩妮</t>
+        </is>
+      </c>
+      <c r="R186" t="inlineStr">
+        <is>
+          <t>Mira</t>
+        </is>
+      </c>
+      <c r="S186" t="inlineStr">
+        <is>
+          <t>ミラ</t>
+        </is>
+      </c>
+      <c r="T186" t="inlineStr">
+        <is>
+          <t>미라</t>
+        </is>
+      </c>
+      <c r="U186" t="inlineStr">
+        <is>
+          <t>米拉</t>
+        </is>
+      </c>
+      <c r="V186" t="inlineStr">
+        <is>
+          <t>米拉</t>
+        </is>
+      </c>
+      <c r="W186" t="inlineStr">
+        <is>
+          <t>DisCoins</t>
+        </is>
+      </c>
+      <c r="X186" t="inlineStr">
+        <is>
+          <t>ディスコイン</t>
+        </is>
+      </c>
+      <c r="Y186" t="inlineStr">
+        <is>
+          <t>디스코인</t>
+        </is>
+      </c>
+      <c r="Z186" t="inlineStr">
+        <is>
+          <t>狄斯币</t>
+        </is>
+      </c>
+      <c r="AA186" t="inlineStr">
+        <is>
+          <t>狄斯幣</t>
+        </is>
+      </c>
+      <c r="AB186" t="inlineStr">
+        <is>
+          <t>4000.0</t>
+        </is>
+      </c>
+      <c r="AC186" t="inlineStr">
+        <is>
+          <t>DisCoins</t>
+        </is>
+      </c>
+      <c r="AD186" t="inlineStr">
+        <is>
+          <t>ディスコイン</t>
+        </is>
+      </c>
+      <c r="AE186" t="inlineStr">
+        <is>
+          <t>디스코인</t>
+        </is>
+      </c>
+      <c r="AF186" t="inlineStr">
+        <is>
+          <t>狄斯币</t>
+        </is>
+      </c>
+      <c r="AG186" t="inlineStr">
+        <is>
+          <t>狄斯幣</t>
+        </is>
+      </c>
+      <c r="AH186" t="inlineStr">
+        <is>
+          <t>1000.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="n">
+        <v>1099001</v>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>Green</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>Dream Interpretation</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>夢の解析</t>
+        </is>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>꿈의 해석</t>
+        </is>
+      </c>
+      <c r="F187" t="inlineStr">
+        <is>
+          <t>梦的解析</t>
+        </is>
+      </c>
+      <c r="G187" t="inlineStr">
+        <is>
+          <t>夢的解析</t>
+        </is>
+      </c>
+      <c r="H187" t="inlineStr">
+        <is>
+          <t>Residents in some areas of Eastside often suffer from nightmares. It is necessary to find out why.</t>
+        </is>
+      </c>
+      <c r="I187" t="inlineStr">
+        <is>
+          <t>ニューシティの一部エリアの住民がよくナイトメアにうなされている。具体的な原因を調査しなければならない。</t>
+        </is>
+      </c>
+      <c r="J187" t="inlineStr">
+        <is>
+          <t>신성 일부 지역 주민들은 악몽을 자주꾼다. 구체적인 원인을 철저히 조사해야 한다.</t>
+        </is>
+      </c>
+      <c r="K187" t="inlineStr">
+        <is>
+          <t>新城一些区域的居民经常做噩梦，需要查清具体原因。</t>
+        </is>
+      </c>
+      <c r="L187" t="inlineStr">
+        <is>
+          <t>新城一些區域的居民經常做惡夢，需要查明具體原因。</t>
+        </is>
+      </c>
+      <c r="M187" t="inlineStr">
+        <is>
+          <t>Hecate</t>
+        </is>
+      </c>
+      <c r="N187" t="inlineStr">
+        <is>
+          <t>ヘカテー</t>
+        </is>
+      </c>
+      <c r="O187" t="inlineStr">
+        <is>
+          <t>헤카테</t>
+        </is>
+      </c>
+      <c r="P187" t="inlineStr">
+        <is>
+          <t>赫卡蒂</t>
+        </is>
+      </c>
+      <c r="Q187" t="inlineStr">
+        <is>
+          <t>赫卡蒂</t>
+        </is>
+      </c>
+      <c r="R187" t="inlineStr"/>
+      <c r="S187" t="inlineStr"/>
+      <c r="T187" t="inlineStr"/>
+      <c r="U187" t="inlineStr"/>
+      <c r="V187" t="inlineStr"/>
+      <c r="W187" t="inlineStr">
+        <is>
           <t>Arsenopyrite Concentrate</t>
         </is>
       </c>
-      <c r="X181" t="inlineStr">
+      <c r="X187" t="inlineStr">
         <is>
           <t>毒砂の精鉱</t>
         </is>
       </c>
-      <c r="Y181" t="inlineStr">
+      <c r="Y187" t="inlineStr">
         <is>
           <t>정교한 독모래 광석</t>
         </is>
       </c>
-      <c r="Z181" t="inlineStr">
+      <c r="Z187" t="inlineStr">
         <is>
           <t>毒砂精矿</t>
         </is>
       </c>
-      <c r="AA181" t="inlineStr">
+      <c r="AA187" t="inlineStr">
         <is>
           <t>毒砂精礦</t>
         </is>
       </c>
-      <c r="AB181" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="AC181" t="inlineStr">
+      <c r="AB187" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AC187" t="inlineStr">
         <is>
           <t>Arsenopyrite Raw Ore</t>
         </is>
       </c>
-      <c r="AD181" t="inlineStr">
+      <c r="AD187" t="inlineStr">
         <is>
           <t>毒砂の原鉱</t>
         </is>
       </c>
-      <c r="AE181" t="inlineStr">
+      <c r="AE187" t="inlineStr">
         <is>
           <t>거친 독모래 광석</t>
         </is>
       </c>
-      <c r="AF181" t="inlineStr">
+      <c r="AF187" t="inlineStr">
         <is>
           <t>毒砂粗矿</t>
         </is>
       </c>
-      <c r="AG181" t="inlineStr">
+      <c r="AG187" t="inlineStr">
         <is>
           <t>毒砂粗礦</t>
         </is>
       </c>
-      <c r="AH181" t="inlineStr">
+      <c r="AH187" t="inlineStr">
         <is>
           <t>1.0</t>
         </is>

</xml_diff>

<commit_message>
GLB - Ceto Update
</commit_message>
<xml_diff>
--- a/Sinner_Stuff/dispatch.xlsx
+++ b/Sinner_Stuff/dispatch.xlsx
@@ -27453,7 +27453,7 @@
       </c>
       <c r="J174" t="inlineStr">
         <is>
-          <t>정보원에 따르면 신성의 어느 한 부자가 암암리에 변이 무기 밀수 조직을 지원한다고 한다. 이에 따라 관리국은 작전 요원을 해당 인물의 사교계에 잠입시켜 조사를 진행할 예정이며, 현재 상류층 내에서 명망 있는 인물의 소개가 필요한 상황이다.</t>
+          <t>정보원에 따르면 신성의 어느 한 부자가 암암리에 변이 무기 밀수 조직을 지원한다고 한다. 이에 따라 관리국은 작전요원을 해당 인물의 사교계에 잠입시켜 조사를 진행할 예정이며, 현재 상류층 내에서 명망 있는 인물의 소개가 필요한 상황이다.</t>
         </is>
       </c>
       <c r="K174" t="inlineStr">
@@ -27603,7 +27603,7 @@
       </c>
       <c r="J175" t="inlineStr">
         <is>
-          <t>최근 신성에서 무용 대회를 개최하고 있다. 대회 시작 이후 경기장 내 M 수치가 지속적으로 비정상적인 파동을 보이고 있다. 이에 FAC는 관리국에 무용에 능한 수감자를 파견해 작전 요원과 함께 잠입 조사를 해달라고 요청했다.</t>
+          <t>최근 신성에서 무용 대회를 개최하고 있다. 대회 시작 이후 경기장 내 M 수치가 지속적으로 비정상적인 파동을 보이고 있다. 이에 FAC는 관리국에 무용에 능한 수감자를 파견해 작전요원과 함께 잠입 조사를 해달라고 요청했다.</t>
         </is>
       </c>
       <c r="K175" t="inlineStr">
@@ -28983,12 +28983,12 @@
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>###</t>
+          <t>サーカスの疑惑</t>
         </is>
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>###</t>
+          <t>서커스단 의문점</t>
         </is>
       </c>
       <c r="F184" t="inlineStr">
@@ -29008,12 +29008,12 @@
       </c>
       <c r="I184" t="inlineStr">
         <is>
-          <t>###</t>
+          <t>最近、ニューシティの有名なサーカス団に虐待スキャンダルが持ち上がった。潜入調査を行うため、治安局は実力が高く、風変わりな外見のコンビクトを一名緊急募集している。</t>
         </is>
       </c>
       <c r="J184" t="inlineStr">
         <is>
-          <t>###</t>
+          <t>최근 신성의 한 유명 서커스단에서 학대 스캔들이 터져 나왔다. 치안국에서 실력이 강하고, 외모가 평범하지 않은 수감자가 지원해 잠입 조사를 도와주기를 기다리고 있다.</t>
         </is>
       </c>
       <c r="K184" t="inlineStr">
@@ -29133,12 +29133,12 @@
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>###</t>
+          <t>広場の清掃</t>
         </is>
       </c>
       <c r="E185" t="inlineStr">
         <is>
-          <t>###</t>
+          <t>광장 청소</t>
         </is>
       </c>
       <c r="F185" t="inlineStr">
@@ -29158,12 +29158,12 @@
       </c>
       <c r="I185" t="inlineStr">
         <is>
-          <t>###</t>
+          <t>祝賀行事の期間中は出かける人が多すぎるため、広場の清掃を担当する清掃部門の人手が不足する。雑務に長けたコンビクトを作業に参加させることが急務だ。</t>
         </is>
       </c>
       <c r="J185" t="inlineStr">
         <is>
-          <t>###</t>
+          <t>축제 기간, 찾아오는 사람이 너무 많아져서, 광장 청소를 맡은 환경미화 부서의 일손이 부족해졌다. 환경미화 부서를 돕기 위해 잡일에 능한 수감자를 파견해야 한다.</t>
         </is>
       </c>
       <c r="K185" t="inlineStr">
@@ -29183,7 +29183,7 @@
       </c>
       <c r="N185" t="inlineStr">
         <is>
-          <t>###</t>
+          <t>サニー</t>
         </is>
       </c>
       <c r="O185" t="inlineStr">
@@ -29283,12 +29283,12 @@
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>###</t>
+          <t>変装して潜入</t>
         </is>
       </c>
       <c r="E186" t="inlineStr">
         <is>
-          <t>###</t>
+          <t>위장 잠입</t>
         </is>
       </c>
       <c r="F186" t="inlineStr">
@@ -29308,12 +29308,12 @@
       </c>
       <c r="I186" t="inlineStr">
         <is>
-          <t>###</t>
+          <t>最新の情報によると、ニューシティのとあるホテルで人質事件が発生したという。人質の安全を確保するため、コンビクト二名を緊急手配し、従業員に変装させて現場に潜入させる必要がある。</t>
         </is>
       </c>
       <c r="J186" t="inlineStr">
         <is>
-          <t>###</t>
+          <t>최신 소식에 따르면 신성의 한 호텔에서 인질극이 발생했다고 한다. 인질을 보호하기 위해, 수감자 두 명을 긴급하게 파견해 종업원으로 위장해 현장에 잠입시켜야 한다.</t>
         </is>
       </c>
       <c r="K186" t="inlineStr">
@@ -29333,7 +29333,7 @@
       </c>
       <c r="N186" t="inlineStr">
         <is>
-          <t>###</t>
+          <t>サニー</t>
         </is>
       </c>
       <c r="O186" t="inlineStr">
@@ -29439,86 +29439,86 @@
     </row>
     <row r="187">
       <c r="A187" t="n">
-        <v>1099001</v>
+        <v>1058001</v>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>Green</t>
+          <t>Purple</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>Dream Interpretation</t>
+          <t>Strategic Coordination</t>
         </is>
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>夢の解析</t>
+          <t>戦術統括</t>
         </is>
       </c>
       <c r="E187" t="inlineStr">
         <is>
-          <t>꿈의 해석</t>
+          <t>전술 총괄</t>
         </is>
       </c>
       <c r="F187" t="inlineStr">
         <is>
-          <t>梦的解析</t>
+          <t>战术统筹</t>
         </is>
       </c>
       <c r="G187" t="inlineStr">
         <is>
-          <t>夢的解析</t>
+          <t>戰術統籌</t>
         </is>
       </c>
       <c r="H187" t="inlineStr">
         <is>
-          <t>Residents in some areas of Eastside often suffer from nightmares. It is necessary to find out why.</t>
+          <t>There has been a recent surge of Corruptors near the Rust and the situation is dire. We urgently need a Sinner with experience in strategic planning and battlefield command to serve as the Acting Commander and coordinate the operations.</t>
         </is>
       </c>
       <c r="I187" t="inlineStr">
         <is>
-          <t>ニューシティの一部エリアの住民がよくナイトメアにうなされている。具体的な原因を調査しなければならない。</t>
+          <t>錆の川地帯では近頃、死瞳が急増し緊迫した状況だ。直ちに全体的な統括と実戦指揮の経験を持つコンビクトを派遣し、臨時の作戦総指揮として作戦全体を調整する必要がある。</t>
         </is>
       </c>
       <c r="J187" t="inlineStr">
         <is>
-          <t>신성 일부 지역 주민들은 악몽을 자주꾼다. 구체적인 원인을 철저히 조사해야 한다.</t>
+          <t>러스트 리버 지대에서 최근 괴변체가 급증하여 상황이 긴박해졌다. 현재 급히 전반적인 상황을 통솔하고 실전 지휘가 풍부한 수감자를 파견해 작전 총지휘를 맡기고 전체 작전을 조율해야 한다.</t>
         </is>
       </c>
       <c r="K187" t="inlineStr">
         <is>
-          <t>新城一些区域的居民经常做噩梦，需要查清具体原因。</t>
+          <t>锈河地带近日死役激增，局势紧张，当下急需一位具备全局统筹与实战指挥经验的禁闭者前往，临时担任作战总指挥，协调整体行动。</t>
         </is>
       </c>
       <c r="L187" t="inlineStr">
         <is>
-          <t>新城一些區域的居民經常做惡夢，需要查明具體原因。</t>
+          <t>鏽河地帶近日死役激增，局勢緊張，當下急需一位具備全局統籌與實戰指揮經驗的禁閉者前往，臨時擔任作戰總指揮，協調整體行動。</t>
         </is>
       </c>
       <c r="M187" t="inlineStr">
         <is>
-          <t>Hecate</t>
+          <t>Augustus</t>
         </is>
       </c>
       <c r="N187" t="inlineStr">
         <is>
-          <t>ヘカテー</t>
+          <t>アウグスタ</t>
         </is>
       </c>
       <c r="O187" t="inlineStr">
         <is>
-          <t>헤카테</t>
+          <t>아우구스트</t>
         </is>
       </c>
       <c r="P187" t="inlineStr">
         <is>
-          <t>赫卡蒂</t>
+          <t>奥古斯特</t>
         </is>
       </c>
       <c r="Q187" t="inlineStr">
         <is>
-          <t>赫卡蒂</t>
+          <t>奧古斯特</t>
         </is>
       </c>
       <c r="R187" t="inlineStr"/>
@@ -29528,60 +29528,1150 @@
       <c r="V187" t="inlineStr"/>
       <c r="W187" t="inlineStr">
         <is>
+          <t>Mania Essence</t>
+        </is>
+      </c>
+      <c r="X187" t="inlineStr">
+        <is>
+          <t>ルナティックエッセンス</t>
+        </is>
+      </c>
+      <c r="Y187" t="inlineStr">
+        <is>
+          <t>광란의 정수</t>
+        </is>
+      </c>
+      <c r="Z187" t="inlineStr">
+        <is>
+          <t>狂乱精粹</t>
+        </is>
+      </c>
+      <c r="AA187" t="inlineStr">
+        <is>
+          <t>狂亂精粹</t>
+        </is>
+      </c>
+      <c r="AB187" t="inlineStr">
+        <is>
+          <t>8000.0</t>
+        </is>
+      </c>
+      <c r="AC187" t="inlineStr">
+        <is>
+          <t>Mania Essence</t>
+        </is>
+      </c>
+      <c r="AD187" t="inlineStr">
+        <is>
+          <t>ルナティックエッセンス</t>
+        </is>
+      </c>
+      <c r="AE187" t="inlineStr">
+        <is>
+          <t>광란의 정수</t>
+        </is>
+      </c>
+      <c r="AF187" t="inlineStr">
+        <is>
+          <t>狂乱精粹</t>
+        </is>
+      </c>
+      <c r="AG187" t="inlineStr">
+        <is>
+          <t>狂亂精粹</t>
+        </is>
+      </c>
+      <c r="AH187" t="inlineStr">
+        <is>
+          <t>2000.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="n">
+        <v>1058002</v>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>Purple</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>Justified Force</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>拳に理あり</t>
+        </is>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>정당한 주먹</t>
+        </is>
+      </c>
+      <c r="F188" t="inlineStr">
+        <is>
+          <t>出拳有理</t>
+        </is>
+      </c>
+      <c r="G188" t="inlineStr">
+        <is>
+          <t>出拳有理</t>
+        </is>
+      </c>
+      <c r="H188" t="inlineStr">
+        <is>
+          <t>Reports of thugs terrorizing civilians have become frequent in a certain neighborhood in Syndicate. A recent incident involving injured children has even sparked public outrage. The news has rendered a certain Sinner furious, who insists on intervening to uphold justice and protect vulnerable individuals.</t>
+        </is>
+      </c>
+      <c r="I188" t="inlineStr">
+        <is>
+          <t>シンジケートの一角で悪党が平民を虐げる事案が頻発している。近頃は子供が負傷する事件も発生し、市民の怒りを買っている状況だ。これを聞いて激怒したあるコンビクトが、正義を守り弱者の安全を保護するために出撃を強く求めた。</t>
+        </is>
+      </c>
+      <c r="J188" t="inlineStr">
+        <is>
+          <t>신디케이트의 어느 디스트릭트에서 악당들이 일반인을 괴롭힌다는 제보가 잇따르고 있고, 최근에는 아이가 다치는 사건까지 발생해 민중들의 공분을 사게 됐다. 소식을 들은 어느 수감자는 매우 분노하며, 정의를 지키고 약자를 보호하겠다고 강력하게 주장했다.</t>
+        </is>
+      </c>
+      <c r="K188" t="inlineStr">
+        <is>
+          <t>辛迪加一街区频传恶徒欺压平民之事，近日更有孩童受伤事件引发民愤。某禁闭者得知消息后怒不可遏，强烈要求出手维护正义，保护弱者安全。</t>
+        </is>
+      </c>
+      <c r="L188" t="inlineStr">
+        <is>
+          <t>辛迪加一街區頻傳惡徒欺壓平民之事，近日更有孩童受傷事件引發民憤。某禁閉者得知消息後怒不可遏，強烈要求出手維護正義，保護弱者安全。</t>
+        </is>
+      </c>
+      <c r="M188" t="inlineStr">
+        <is>
+          <t>Necresta·Hella</t>
+        </is>
+      </c>
+      <c r="N188" t="inlineStr">
+        <is>
+          <t>幽冠・ヘラ</t>
+        </is>
+      </c>
+      <c r="O188" t="inlineStr">
+        <is>
+          <t>유혼·엘라</t>
+        </is>
+      </c>
+      <c r="P188" t="inlineStr">
+        <is>
+          <t>幽冕·海拉</t>
+        </is>
+      </c>
+      <c r="Q188" t="inlineStr">
+        <is>
+          <t>幽冕·海拉</t>
+        </is>
+      </c>
+      <c r="R188" t="inlineStr"/>
+      <c r="S188" t="inlineStr"/>
+      <c r="T188" t="inlineStr"/>
+      <c r="U188" t="inlineStr"/>
+      <c r="V188" t="inlineStr"/>
+      <c r="W188" t="inlineStr">
+        <is>
+          <t>Mania Essence</t>
+        </is>
+      </c>
+      <c r="X188" t="inlineStr">
+        <is>
+          <t>ルナティックエッセンス</t>
+        </is>
+      </c>
+      <c r="Y188" t="inlineStr">
+        <is>
+          <t>광란의 정수</t>
+        </is>
+      </c>
+      <c r="Z188" t="inlineStr">
+        <is>
+          <t>狂乱精粹</t>
+        </is>
+      </c>
+      <c r="AA188" t="inlineStr">
+        <is>
+          <t>狂亂精粹</t>
+        </is>
+      </c>
+      <c r="AB188" t="inlineStr">
+        <is>
+          <t>8000.0</t>
+        </is>
+      </c>
+      <c r="AC188" t="inlineStr">
+        <is>
+          <t>Mania Essence</t>
+        </is>
+      </c>
+      <c r="AD188" t="inlineStr">
+        <is>
+          <t>ルナティックエッセンス</t>
+        </is>
+      </c>
+      <c r="AE188" t="inlineStr">
+        <is>
+          <t>광란의 정수</t>
+        </is>
+      </c>
+      <c r="AF188" t="inlineStr">
+        <is>
+          <t>狂乱精粹</t>
+        </is>
+      </c>
+      <c r="AG188" t="inlineStr">
+        <is>
+          <t>狂亂精粹</t>
+        </is>
+      </c>
+      <c r="AH188" t="inlineStr">
+        <is>
+          <t>2000.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="n">
+        <v>1058003</v>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>Green</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>Communication Blackout Crisis</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>通信切断危機</t>
+        </is>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>통신 두절 위기</t>
+        </is>
+      </c>
+      <c r="F189" t="inlineStr">
+        <is>
+          <t>断讯危机</t>
+        </is>
+      </c>
+      <c r="G189" t="inlineStr">
+        <is>
+          <t>斷訊危機</t>
+        </is>
+      </c>
+      <c r="H189" t="inlineStr">
+        <is>
+          <t>Multiple signal towers in Eastside have been deliberately sabotaged, causing a communication blackout in the area. The Public Security Bureau has submitted an urgent request to the MBCC to dispatch a Sinner with extensive knowledge of signal tower structures and communication systems to assist with emergency repairs and apprehend the perpetrators.</t>
+        </is>
+      </c>
+      <c r="I189" t="inlineStr">
+        <is>
+          <t>ニューシティの複数の電波塔が人為的に破壊され、地域の通信が切断されてしまった。治安局は管理局に緊急要請を行い、電波塔の構造や通信機構に精通したコンビクトを派遣し、設備の修復および犯人の調査に協力することを求めている。</t>
+        </is>
+      </c>
+      <c r="J189" t="inlineStr">
+        <is>
+          <t>신성의 여러 통신 탑이 파괴되어, 일부 지역의 통신이 두절되었다. 치안국은 관리국에 통신 탑의 구조와 통신 메커니즘에 대해 깊은 이해도를 갖춘 수감자를 파견하여 범인을 찾고 장비를 복구할 수 있도록 도움을 요청했다.</t>
+        </is>
+      </c>
+      <c r="K189" t="inlineStr">
+        <is>
+          <t>新城的多座信号塔遭遇人为破坏，造成片区通信中断。治安局向管理局提出紧急申请，需派遣一位对信号塔结构与通讯机制有深入了解的禁闭者，协助抢修设备、调查元凶。</t>
+        </is>
+      </c>
+      <c r="L189" t="inlineStr">
+        <is>
+          <t>新城的多座訊號塔遭到人為破壞，造成片區通訊中斷。治安局向管理局提出緊急申請，需派遣一位對訊號塔結構與通訊機制有深入瞭解的禁閉者，協助搶修設備、調查元凶。</t>
+        </is>
+      </c>
+      <c r="M189" t="inlineStr">
+        <is>
+          <t>Siglinde</t>
+        </is>
+      </c>
+      <c r="N189" t="inlineStr">
+        <is>
+          <t>ジークリンデ</t>
+        </is>
+      </c>
+      <c r="O189" t="inlineStr">
+        <is>
+          <t>시글린데</t>
+        </is>
+      </c>
+      <c r="P189" t="inlineStr">
+        <is>
+          <t>希格林德</t>
+        </is>
+      </c>
+      <c r="Q189" t="inlineStr">
+        <is>
+          <t>希格林德</t>
+        </is>
+      </c>
+      <c r="R189" t="inlineStr"/>
+      <c r="S189" t="inlineStr"/>
+      <c r="T189" t="inlineStr"/>
+      <c r="U189" t="inlineStr"/>
+      <c r="V189" t="inlineStr"/>
+      <c r="W189" t="inlineStr">
+        <is>
+          <t>Mania Essence</t>
+        </is>
+      </c>
+      <c r="X189" t="inlineStr">
+        <is>
+          <t>ルナティックエッセンス</t>
+        </is>
+      </c>
+      <c r="Y189" t="inlineStr">
+        <is>
+          <t>광란의 정수</t>
+        </is>
+      </c>
+      <c r="Z189" t="inlineStr">
+        <is>
+          <t>狂乱精粹</t>
+        </is>
+      </c>
+      <c r="AA189" t="inlineStr">
+        <is>
+          <t>狂亂精粹</t>
+        </is>
+      </c>
+      <c r="AB189" t="inlineStr">
+        <is>
+          <t>2400.0</t>
+        </is>
+      </c>
+      <c r="AC189" t="inlineStr">
+        <is>
+          <t>Mania Essence</t>
+        </is>
+      </c>
+      <c r="AD189" t="inlineStr">
+        <is>
+          <t>ルナティックエッセンス</t>
+        </is>
+      </c>
+      <c r="AE189" t="inlineStr">
+        <is>
+          <t>광란의 정수</t>
+        </is>
+      </c>
+      <c r="AF189" t="inlineStr">
+        <is>
+          <t>狂乱精粹</t>
+        </is>
+      </c>
+      <c r="AG189" t="inlineStr">
+        <is>
+          <t>狂亂精粹</t>
+        </is>
+      </c>
+      <c r="AH189" t="inlineStr">
+        <is>
+          <t>800.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="n">
+        <v>1058004</v>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>Blue</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>Commercial Mediation</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>商業エリアのブレークポイント</t>
+        </is>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>상권 분리 지점</t>
+        </is>
+      </c>
+      <c r="F190" t="inlineStr">
+        <is>
+          <t>商圈断点</t>
+        </is>
+      </c>
+      <c r="G190" t="inlineStr">
+        <is>
+          <t>商圈斷點</t>
+        </is>
+      </c>
+      <c r="H190" t="inlineStr">
+        <is>
+          <t>Two major corporations in Eastside are in conflict over the planning of a certain urban area, affecting business partners and nearby residential areas. The Bureau has decided to send someone skilled in negotiation to mediate on-site, preventing the situation from escalating further.</t>
+        </is>
+      </c>
+      <c r="I190" t="inlineStr">
+        <is>
+          <t>ニューシティの二大企業が通りに面した区画計画を巡って対立しており、その衝突が協力会社や近隣住民区にまで及んでいる。管理局は調停に長けた人員を現地に派遣し、交渉に介入して事態のさらなる拡大を防ぐことを決定した。</t>
+        </is>
+      </c>
+      <c r="J190" t="inlineStr">
+        <is>
+          <t>신성의 두 대기업이 도로 접경지의 개발로 인해 충돌하면서, 이들의 갈등은 협력업체와 주변 주거 구역까지 확산했다. 관리국에서는 협상에 능한 인원을 현장에 파견하여, 사태 확산을 막기 위해 중재하기로 했다.</t>
+        </is>
+      </c>
+      <c r="K190" t="inlineStr">
+        <is>
+          <t>新城两家大型企业因临街地块规划发生冲突，矛盾已蔓延至合作商与附近居民区。管理局决定派擅长协调交涉的人员前往现场，介入调解，防止事态进一步升级。</t>
+        </is>
+      </c>
+      <c r="L190" t="inlineStr">
+        <is>
+          <t>新城兩家大型企業因臨街地塊規劃發生衝突，矛盾已蔓延至合作商與附近住宅區。管理局決定派擅長協調交涉的人員前往現場，介入調解，防止事態進一步升級。</t>
+        </is>
+      </c>
+      <c r="M190" t="inlineStr">
+        <is>
+          <t>Siglinde</t>
+        </is>
+      </c>
+      <c r="N190" t="inlineStr">
+        <is>
+          <t>ジークリンデ</t>
+        </is>
+      </c>
+      <c r="O190" t="inlineStr">
+        <is>
+          <t>시글린데</t>
+        </is>
+      </c>
+      <c r="P190" t="inlineStr">
+        <is>
+          <t>希格林德</t>
+        </is>
+      </c>
+      <c r="Q190" t="inlineStr">
+        <is>
+          <t>希格林德</t>
+        </is>
+      </c>
+      <c r="R190" t="inlineStr">
+        <is>
+          <t>Mr. Fox</t>
+        </is>
+      </c>
+      <c r="S190" t="inlineStr">
+        <is>
+          <t>Mr.Fox</t>
+        </is>
+      </c>
+      <c r="T190" t="inlineStr">
+        <is>
+          <t>Mr.Fox</t>
+        </is>
+      </c>
+      <c r="U190" t="inlineStr">
+        <is>
+          <t>福克斯先生</t>
+        </is>
+      </c>
+      <c r="V190" t="inlineStr">
+        <is>
+          <t>Mr.Fox</t>
+        </is>
+      </c>
+      <c r="W190" t="inlineStr">
+        <is>
+          <t>Mania Essence</t>
+        </is>
+      </c>
+      <c r="X190" t="inlineStr">
+        <is>
+          <t>ルナティックエッセンス</t>
+        </is>
+      </c>
+      <c r="Y190" t="inlineStr">
+        <is>
+          <t>광란의 정수</t>
+        </is>
+      </c>
+      <c r="Z190" t="inlineStr">
+        <is>
+          <t>狂乱精粹</t>
+        </is>
+      </c>
+      <c r="AA190" t="inlineStr">
+        <is>
+          <t>狂亂精粹</t>
+        </is>
+      </c>
+      <c r="AB190" t="inlineStr">
+        <is>
+          <t>4000.0</t>
+        </is>
+      </c>
+      <c r="AC190" t="inlineStr">
+        <is>
+          <t>Mania Essence</t>
+        </is>
+      </c>
+      <c r="AD190" t="inlineStr">
+        <is>
+          <t>ルナティックエッセンス</t>
+        </is>
+      </c>
+      <c r="AE190" t="inlineStr">
+        <is>
+          <t>광란의 정수</t>
+        </is>
+      </c>
+      <c r="AF190" t="inlineStr">
+        <is>
+          <t>狂乱精粹</t>
+        </is>
+      </c>
+      <c r="AG190" t="inlineStr">
+        <is>
+          <t>狂亂精粹</t>
+        </is>
+      </c>
+      <c r="AH190" t="inlineStr">
+        <is>
+          <t>1000.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="n">
+        <v>1059001</v>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>Purple</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>Stormy Invasion</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>嵐襲来</t>
+        </is>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>폭풍의 습격</t>
+        </is>
+      </c>
+      <c r="F191" t="inlineStr">
+        <is>
+          <t>风暴侵袭</t>
+        </is>
+      </c>
+      <c r="G191" t="inlineStr">
+        <is>
+          <t>風暴侵襲</t>
+        </is>
+      </c>
+      <c r="H191" t="inlineStr">
+        <is>
+          <t>A massive storm has struck the border, stranding a shipment of urgently needed rare supplies. We need to recruit a Sinner with experience operating under storms to help escort the cargo and ensure its safety through these extreme weather conditions.</t>
+        </is>
+      </c>
+      <c r="I191" t="inlineStr">
+        <is>
+          <t>辺境が特級の嵐に襲われ、緊急輸送する必要のある希少物資が一部足止めされている。護送を支援し、極端な気象下で物資の安全を確保するため、嵐の環境下での作戦経験があるコンビクトを募集している。</t>
+        </is>
+      </c>
+      <c r="J191" t="inlineStr">
+        <is>
+          <t>국경이 특급 폭풍의 습격을 받아, 국경 안으로 긴급히 운반해야 할 희귀 물자가 멈췄다. 현재 폭풍이 부는 환경에서의 작전 경험을 가진 수감자를 모집해 물자 운송을 돕고, 극한 기상 조건에서 물자의 안전을 보장해야 한다.</t>
+        </is>
+      </c>
+      <c r="K191" t="inlineStr">
+        <is>
+          <t>边境遭特级风暴侵袭，一批急需运入境内的珍稀物资滞留。现需招募具有风暴环境作战经验的禁闭者协助押运，保障物资在极端天气下的安全。</t>
+        </is>
+      </c>
+      <c r="L191" t="inlineStr">
+        <is>
+          <t>邊境遭特級風暴侵襲，一批急需運入境內的珍稀物資滯留。現需招募具有風暴環境作戰經驗的禁閉者協助押運，保障物資在極端天氣下的安全。</t>
+        </is>
+      </c>
+      <c r="M191" t="inlineStr">
+        <is>
+          <t>Ceto</t>
+        </is>
+      </c>
+      <c r="N191" t="inlineStr">
+        <is>
+          <t>セト</t>
+        </is>
+      </c>
+      <c r="O191" t="inlineStr">
+        <is>
+          <t>세토</t>
+        </is>
+      </c>
+      <c r="P191" t="inlineStr">
+        <is>
+          <t>赛托</t>
+        </is>
+      </c>
+      <c r="Q191" t="inlineStr">
+        <is>
+          <t>賽托</t>
+        </is>
+      </c>
+      <c r="R191" t="inlineStr"/>
+      <c r="S191" t="inlineStr"/>
+      <c r="T191" t="inlineStr"/>
+      <c r="U191" t="inlineStr"/>
+      <c r="V191" t="inlineStr"/>
+      <c r="W191" t="inlineStr">
+        <is>
+          <t>Mania Essence</t>
+        </is>
+      </c>
+      <c r="X191" t="inlineStr">
+        <is>
+          <t>ルナティックエッセンス</t>
+        </is>
+      </c>
+      <c r="Y191" t="inlineStr">
+        <is>
+          <t>광란의 정수</t>
+        </is>
+      </c>
+      <c r="Z191" t="inlineStr">
+        <is>
+          <t>狂乱精粹</t>
+        </is>
+      </c>
+      <c r="AA191" t="inlineStr">
+        <is>
+          <t>狂亂精粹</t>
+        </is>
+      </c>
+      <c r="AB191" t="inlineStr">
+        <is>
+          <t>8000.0</t>
+        </is>
+      </c>
+      <c r="AC191" t="inlineStr">
+        <is>
+          <t>Mania Essence</t>
+        </is>
+      </c>
+      <c r="AD191" t="inlineStr">
+        <is>
+          <t>ルナティックエッセンス</t>
+        </is>
+      </c>
+      <c r="AE191" t="inlineStr">
+        <is>
+          <t>광란의 정수</t>
+        </is>
+      </c>
+      <c r="AF191" t="inlineStr">
+        <is>
+          <t>狂乱精粹</t>
+        </is>
+      </c>
+      <c r="AG191" t="inlineStr">
+        <is>
+          <t>狂亂精粹</t>
+        </is>
+      </c>
+      <c r="AH191" t="inlineStr">
+        <is>
+          <t>2000.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="n">
+        <v>1059002</v>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>Green</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>Sand Ship Hijacker</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>砂航船の強盗</t>
+        </is>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>사막 납치범</t>
+        </is>
+      </c>
+      <c r="F192" t="inlineStr">
+        <is>
+          <t>砂船劫匪</t>
+        </is>
+      </c>
+      <c r="G192" t="inlineStr">
+        <is>
+          <t>砂船劫匪</t>
+        </is>
+      </c>
+      <c r="H192" t="inlineStr">
+        <is>
+          <t>Some highly skilled bandits have seized a DisCity sand ship in WhiteSands, demanding that the Public Security Bureau release their accomplices within 8 hours in exchange for the hostages. We urgently need to recruit a Sinner familiar with sand ship layouts who can handle solo combats and react to situations quickly to secretly infiltrate the vessel and safely rescue the hostages.</t>
+        </is>
+      </c>
+      <c r="I192" t="inlineStr">
+        <is>
+          <t>砂の海で、強盗によるディスの砂航船ハイジャック事件が発生した。犯人は治安局に対して、人質と引き換えに8時間以内に仲間を釈放することを要求している。現在、秘密裏に潜入して人質を安全に救出するため、砂航船の内部構造に精通し、単独での戦闘および臨機応変に対応できるコンビクトが1名緊急に必要だ。</t>
+        </is>
+      </c>
+      <c r="J192" t="inlineStr">
+        <is>
+          <t>화이트 샌드의 전문 납치 조직이 디스의 사막 함선을 납치했다. 납치범들은 치안국에 8시간 내에 동료들을 석방하는 조건으로 인질을 교환할 것을 요구했다. 현재 사막 함선의 내부 구조를 잘 알고, 독립 작전과 임기응변에 능한 수감자를 파견해 인질을 안전하게 구출해야 한다.</t>
+        </is>
+      </c>
+      <c r="K192" t="inlineStr">
+        <is>
+          <t>砂海发生职业劫匪劫持狄斯砂船事件，匪徒要求治安局8小时内释放其同伙以交换人质。现急需一名熟悉砂船内部结构、具备独立作战与应变能力的禁闭者，秘密潜入并安全解救人质。</t>
+        </is>
+      </c>
+      <c r="L192" t="inlineStr">
+        <is>
+          <t>砂海發生職業劫匪劫持狄斯砂船事件，匪徒要求治安局8小時內釋放其同夥以交換人質。現急需一名熟悉砂船內部結構、具備獨立作戰與應變能力的禁閉者，秘密潛入並安全解救人質。</t>
+        </is>
+      </c>
+      <c r="M192" t="inlineStr">
+        <is>
+          <t>Ark</t>
+        </is>
+      </c>
+      <c r="N192" t="inlineStr">
+        <is>
+          <t>アーク</t>
+        </is>
+      </c>
+      <c r="O192" t="inlineStr">
+        <is>
+          <t>아크</t>
+        </is>
+      </c>
+      <c r="P192" t="inlineStr">
+        <is>
+          <t>雅可</t>
+        </is>
+      </c>
+      <c r="Q192" t="inlineStr">
+        <is>
+          <t>雅可</t>
+        </is>
+      </c>
+      <c r="R192" t="inlineStr"/>
+      <c r="S192" t="inlineStr"/>
+      <c r="T192" t="inlineStr"/>
+      <c r="U192" t="inlineStr"/>
+      <c r="V192" t="inlineStr"/>
+      <c r="W192" t="inlineStr">
+        <is>
+          <t>Mania Essence</t>
+        </is>
+      </c>
+      <c r="X192" t="inlineStr">
+        <is>
+          <t>ルナティックエッセンス</t>
+        </is>
+      </c>
+      <c r="Y192" t="inlineStr">
+        <is>
+          <t>광란의 정수</t>
+        </is>
+      </c>
+      <c r="Z192" t="inlineStr">
+        <is>
+          <t>狂乱精粹</t>
+        </is>
+      </c>
+      <c r="AA192" t="inlineStr">
+        <is>
+          <t>狂亂精粹</t>
+        </is>
+      </c>
+      <c r="AB192" t="inlineStr">
+        <is>
+          <t>2400.0</t>
+        </is>
+      </c>
+      <c r="AC192" t="inlineStr">
+        <is>
+          <t>Mania Essence</t>
+        </is>
+      </c>
+      <c r="AD192" t="inlineStr">
+        <is>
+          <t>ルナティックエッセンス</t>
+        </is>
+      </c>
+      <c r="AE192" t="inlineStr">
+        <is>
+          <t>광란의 정수</t>
+        </is>
+      </c>
+      <c r="AF192" t="inlineStr">
+        <is>
+          <t>狂乱精粹</t>
+        </is>
+      </c>
+      <c r="AG192" t="inlineStr">
+        <is>
+          <t>狂亂精粹</t>
+        </is>
+      </c>
+      <c r="AH192" t="inlineStr">
+        <is>
+          <t>800.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="n">
+        <v>1059003</v>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>Blue</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>Refugee Resettlement</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>難民の再定住</t>
+        </is>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>유랑민 정착</t>
+        </is>
+      </c>
+      <c r="F193" t="inlineStr">
+        <is>
+          <t>流民安置</t>
+        </is>
+      </c>
+      <c r="G193" t="inlineStr">
+        <is>
+          <t>流民安置</t>
+        </is>
+      </c>
+      <c r="H193" t="inlineStr">
+        <is>
+          <t>DisCity's border control has detained numerous WhiteSands refugees. The language barrier has led to severe communication problems that have escalated to violent confrontations. We urgently need to recruit two Sinners who are fluent in various WhiteSands dialects and empathetic toward refugees to assist with liaison and resettlement.</t>
+        </is>
+      </c>
+      <c r="I193" t="inlineStr">
+        <is>
+          <t>ディスの越境審査機関に砂の海の難民が多数留まっている。方言が多岐に渡るため深刻な意思疎通障害が発生し、武力衝突にまで発展している状況だ。誘導と再定住の支援業務に従事してもらうため、砂の海各地の方言に精通し、難民に共感して接することのできるコンビクトを2名緊急に募集している。</t>
+        </is>
+      </c>
+      <c r="J193" t="inlineStr">
+        <is>
+          <t>디스 입국 관리 기관에서 대량의 화이트 샌드 유랑민이 체류하고 있다. 방언으로 인해 발생한 소통 장애가 무력 충돌로 발전하려고 한다. 현재 화이트 샌드 각 지역의 방언에 능숙하고, 유랑민의 입장을 이해할 수 있는 수감자 2명을 파견해 사태를 수습하고 난민들을 진정시켜야 한다.</t>
+        </is>
+      </c>
+      <c r="K193" t="inlineStr">
+        <is>
+          <t>狄斯入境检查机构滞留大批砂海流民，因口音复杂，引发严重沟通障碍并升级至武力冲突。现紧急招募两名精通砂海各地方言、且对流民抱有同理心的禁闭者，参与疏导与安顿工作。</t>
+        </is>
+      </c>
+      <c r="L193" t="inlineStr">
+        <is>
+          <t>狄斯入境檢查機構滯留大批砂海流民，因口音複雜，引發嚴重溝通障礙並升級至武力衝突。現緊急招募兩名精通砂海各地方言、且對流民抱有同理心的禁閉者，參與疏導與安頓工作。</t>
+        </is>
+      </c>
+      <c r="M193" t="inlineStr">
+        <is>
+          <t>Ark</t>
+        </is>
+      </c>
+      <c r="N193" t="inlineStr">
+        <is>
+          <t>アーク</t>
+        </is>
+      </c>
+      <c r="O193" t="inlineStr">
+        <is>
+          <t>아크</t>
+        </is>
+      </c>
+      <c r="P193" t="inlineStr">
+        <is>
+          <t>雅可</t>
+        </is>
+      </c>
+      <c r="Q193" t="inlineStr">
+        <is>
+          <t>雅可</t>
+        </is>
+      </c>
+      <c r="R193" t="inlineStr">
+        <is>
+          <t>Mira</t>
+        </is>
+      </c>
+      <c r="S193" t="inlineStr">
+        <is>
+          <t>ミラ</t>
+        </is>
+      </c>
+      <c r="T193" t="inlineStr">
+        <is>
+          <t>미라</t>
+        </is>
+      </c>
+      <c r="U193" t="inlineStr">
+        <is>
+          <t>米拉</t>
+        </is>
+      </c>
+      <c r="V193" t="inlineStr">
+        <is>
+          <t>米拉</t>
+        </is>
+      </c>
+      <c r="W193" t="inlineStr">
+        <is>
+          <t>Mania Essence</t>
+        </is>
+      </c>
+      <c r="X193" t="inlineStr">
+        <is>
+          <t>ルナティックエッセンス</t>
+        </is>
+      </c>
+      <c r="Y193" t="inlineStr">
+        <is>
+          <t>광란의 정수</t>
+        </is>
+      </c>
+      <c r="Z193" t="inlineStr">
+        <is>
+          <t>狂乱精粹</t>
+        </is>
+      </c>
+      <c r="AA193" t="inlineStr">
+        <is>
+          <t>狂亂精粹</t>
+        </is>
+      </c>
+      <c r="AB193" t="inlineStr">
+        <is>
+          <t>4000.0</t>
+        </is>
+      </c>
+      <c r="AC193" t="inlineStr">
+        <is>
+          <t>Mania Essence</t>
+        </is>
+      </c>
+      <c r="AD193" t="inlineStr">
+        <is>
+          <t>ルナティックエッセンス</t>
+        </is>
+      </c>
+      <c r="AE193" t="inlineStr">
+        <is>
+          <t>광란의 정수</t>
+        </is>
+      </c>
+      <c r="AF193" t="inlineStr">
+        <is>
+          <t>狂乱精粹</t>
+        </is>
+      </c>
+      <c r="AG193" t="inlineStr">
+        <is>
+          <t>狂亂精粹</t>
+        </is>
+      </c>
+      <c r="AH193" t="inlineStr">
+        <is>
+          <t>1000.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="n">
+        <v>1099001</v>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>Green</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>Dream Interpretation</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>夢の解析</t>
+        </is>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>꿈의 해석</t>
+        </is>
+      </c>
+      <c r="F194" t="inlineStr">
+        <is>
+          <t>梦的解析</t>
+        </is>
+      </c>
+      <c r="G194" t="inlineStr">
+        <is>
+          <t>夢的解析</t>
+        </is>
+      </c>
+      <c r="H194" t="inlineStr">
+        <is>
+          <t>Residents in some areas of Eastside often suffer from nightmares. It is necessary to find out why.</t>
+        </is>
+      </c>
+      <c r="I194" t="inlineStr">
+        <is>
+          <t>ニューシティの一部エリアの住民がよくナイトメアにうなされている。具体的な原因を調査しなければならない。</t>
+        </is>
+      </c>
+      <c r="J194" t="inlineStr">
+        <is>
+          <t>신성 일부 지역 주민들은 악몽을 자주꾼다. 구체적인 원인을 철저히 조사해야 한다.</t>
+        </is>
+      </c>
+      <c r="K194" t="inlineStr">
+        <is>
+          <t>新城一些区域的居民经常做噩梦，需要查清具体原因。</t>
+        </is>
+      </c>
+      <c r="L194" t="inlineStr">
+        <is>
+          <t>新城一些區域的居民經常做惡夢，需要查明具體原因。</t>
+        </is>
+      </c>
+      <c r="M194" t="inlineStr">
+        <is>
+          <t>Hecate</t>
+        </is>
+      </c>
+      <c r="N194" t="inlineStr">
+        <is>
+          <t>ヘカテー</t>
+        </is>
+      </c>
+      <c r="O194" t="inlineStr">
+        <is>
+          <t>헤카테</t>
+        </is>
+      </c>
+      <c r="P194" t="inlineStr">
+        <is>
+          <t>赫卡蒂</t>
+        </is>
+      </c>
+      <c r="Q194" t="inlineStr">
+        <is>
+          <t>赫卡蒂</t>
+        </is>
+      </c>
+      <c r="R194" t="inlineStr"/>
+      <c r="S194" t="inlineStr"/>
+      <c r="T194" t="inlineStr"/>
+      <c r="U194" t="inlineStr"/>
+      <c r="V194" t="inlineStr"/>
+      <c r="W194" t="inlineStr">
+        <is>
           <t>Arsenopyrite Concentrate</t>
         </is>
       </c>
-      <c r="X187" t="inlineStr">
+      <c r="X194" t="inlineStr">
         <is>
           <t>毒砂の精鉱</t>
         </is>
       </c>
-      <c r="Y187" t="inlineStr">
+      <c r="Y194" t="inlineStr">
         <is>
           <t>정교한 독모래 광석</t>
         </is>
       </c>
-      <c r="Z187" t="inlineStr">
+      <c r="Z194" t="inlineStr">
         <is>
           <t>毒砂精矿</t>
         </is>
       </c>
-      <c r="AA187" t="inlineStr">
+      <c r="AA194" t="inlineStr">
         <is>
           <t>毒砂精礦</t>
         </is>
       </c>
-      <c r="AB187" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="AC187" t="inlineStr">
+      <c r="AB194" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AC194" t="inlineStr">
         <is>
           <t>Arsenopyrite Raw Ore</t>
         </is>
       </c>
-      <c r="AD187" t="inlineStr">
+      <c r="AD194" t="inlineStr">
         <is>
           <t>毒砂の原鉱</t>
         </is>
       </c>
-      <c r="AE187" t="inlineStr">
+      <c r="AE194" t="inlineStr">
         <is>
           <t>거친 독모래 광석</t>
         </is>
       </c>
-      <c r="AF187" t="inlineStr">
+      <c r="AF194" t="inlineStr">
         <is>
           <t>毒砂粗矿</t>
         </is>
       </c>
-      <c r="AG187" t="inlineStr">
+      <c r="AG194" t="inlineStr">
         <is>
           <t>毒砂粗礦</t>
         </is>
       </c>
-      <c r="AH187" t="inlineStr">
+      <c r="AH194" t="inlineStr">
         <is>
           <t>1.0</t>
         </is>

</xml_diff>

<commit_message>
GLB - 20260408 Lichen Event Update
</commit_message>
<xml_diff>
--- a/Sinner_Stuff/dispatch.xlsx
+++ b/Sinner_Stuff/dispatch.xlsx
@@ -30529,86 +30529,86 @@
     </row>
     <row r="194">
       <c r="A194" t="n">
-        <v>1099001</v>
+        <v>1060001</v>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>Green</t>
+          <t>Purple</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>Dream Interpretation</t>
+          <t>Encrypted Radio</t>
         </is>
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>夢の解析</t>
+          <t>暗号化ラジオ</t>
         </is>
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t>꿈의 해석</t>
+          <t>암호화된 라디오</t>
         </is>
       </c>
       <c r="F194" t="inlineStr">
         <is>
-          <t>梦的解析</t>
+          <t>加密电台</t>
         </is>
       </c>
       <c r="G194" t="inlineStr">
         <is>
-          <t>夢的解析</t>
+          <t>加密電台</t>
         </is>
       </c>
       <c r="H194" t="inlineStr">
         <is>
-          <t>Residents in some areas of Eastside often suffer from nightmares. It is necessary to find out why.</t>
+          <t>A mysterious, unregistered radio signal has begun transmitting across the urban district, its broadcast consisting of nothing but sequences of random numbers. The Public Security Bureau fears this may be a new form of encrypted communication. To contain the potential risk, they are urgently recruiting a skilled cryptographer to aid in the decoding operation.</t>
         </is>
       </c>
       <c r="I194" t="inlineStr">
         <is>
-          <t>ニューシティの一部エリアの住民がよくナイトメアにうなされている。具体的な原因を調査しなければならない。</t>
+          <t>都市内で正体不明のラジオが突然現れ、意味不明な数字列を延々と放送している。治安局はこれを新型暗号通信であると疑い、潜在的脅威の拡大を防ぐため、暗号解読に精通した専門家を1名募集し、支援にあたらせるつもりだ。</t>
         </is>
       </c>
       <c r="J194" t="inlineStr">
         <is>
-          <t>신성 일부 지역 주민들은 악몽을 자주꾼다. 구체적인 원인을 철저히 조사해야 한다.</t>
+          <t>도시에 갑자기 정체불명의 라디오가 나타나, 의미를 알 수 없는 숫자를 줄지어 송출하고 있다. 치안국은 이 신호가 새로운 통신 암호문일 것으로 의심하고 있으며, 잠재적 위협의 확산을 막기 위해 암호 해독 전문가 한 명의 지원을 요청했다.</t>
         </is>
       </c>
       <c r="K194" t="inlineStr">
         <is>
-          <t>新城一些区域的居民经常做噩梦，需要查清具体原因。</t>
+          <t>城区内突现不明电台，持续播送成串无意义的数字广播。治安局怀疑该信号为新式通信密文，为防止潜在威胁扩大，现招募一名精通密码破译的专家前往支援。</t>
         </is>
       </c>
       <c r="L194" t="inlineStr">
         <is>
-          <t>新城一些區域的居民經常做惡夢，需要查明具體原因。</t>
+          <t>城區內突現不明電台，持續播送成串無意義的數位廣播。治安局懷疑該訊號為新式通訊密文，為防止潛在威脅擴大，現招募一名精通密碼破譯的專家前往支援。</t>
         </is>
       </c>
       <c r="M194" t="inlineStr">
         <is>
-          <t>Hecate</t>
+          <t>Hilda</t>
         </is>
       </c>
       <c r="N194" t="inlineStr">
         <is>
-          <t>ヘカテー</t>
+          <t>ヒルダ</t>
         </is>
       </c>
       <c r="O194" t="inlineStr">
         <is>
-          <t>헤카테</t>
+          <t>힐다</t>
         </is>
       </c>
       <c r="P194" t="inlineStr">
         <is>
-          <t>赫卡蒂</t>
+          <t>希露妲</t>
         </is>
       </c>
       <c r="Q194" t="inlineStr">
         <is>
-          <t>赫卡蒂</t>
+          <t>希露妲</t>
         </is>
       </c>
       <c r="R194" t="inlineStr"/>
@@ -30618,60 +30618,1450 @@
       <c r="V194" t="inlineStr"/>
       <c r="W194" t="inlineStr">
         <is>
+          <t>Hypercube</t>
+        </is>
+      </c>
+      <c r="X194" t="inlineStr">
+        <is>
+          <t>イレギュラーキューブ</t>
+        </is>
+      </c>
+      <c r="Y194" t="inlineStr">
+        <is>
+          <t>큐브</t>
+        </is>
+      </c>
+      <c r="Z194" t="inlineStr">
+        <is>
+          <t>异方晶</t>
+        </is>
+      </c>
+      <c r="AA194" t="inlineStr">
+        <is>
+          <t>異方晶</t>
+        </is>
+      </c>
+      <c r="AB194" t="inlineStr">
+        <is>
+          <t>30.0</t>
+        </is>
+      </c>
+      <c r="AC194" t="inlineStr">
+        <is>
+          <t>Hypercube</t>
+        </is>
+      </c>
+      <c r="AD194" t="inlineStr">
+        <is>
+          <t>イレギュラーキューブ</t>
+        </is>
+      </c>
+      <c r="AE194" t="inlineStr">
+        <is>
+          <t>큐브</t>
+        </is>
+      </c>
+      <c r="AF194" t="inlineStr">
+        <is>
+          <t>异方晶</t>
+        </is>
+      </c>
+      <c r="AG194" t="inlineStr">
+        <is>
+          <t>異方晶</t>
+        </is>
+      </c>
+      <c r="AH194" t="inlineStr">
+        <is>
+          <t>10.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="n">
+        <v>1061001</v>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>Purple</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>Smash Hit Series</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>人気撮影</t>
+        </is>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>히트작 촬영</t>
+        </is>
+      </c>
+      <c r="F195" t="inlineStr">
+        <is>
+          <t>爆款拍摄</t>
+        </is>
+      </c>
+      <c r="G195" t="inlineStr">
+        <is>
+          <t>爆紅拍攝</t>
+        </is>
+      </c>
+      <c r="H195" t="inlineStr">
+        <is>
+          <t>Some Sinners have formed a mini-series production crew in the Bureau and are now recruiting Sinners with strong writing skills to help craft scripts full of dramatic twists and intense conflicts.</t>
+        </is>
+      </c>
+      <c r="I195" t="inlineStr">
+        <is>
+          <t>管理局内の一部コンビクトが自主的にショートドラマ撮影チームを結成した。波乱万丈で火花が散るようなストーリー展開を作るため、現在脚本に長けたコンビクトを募集している。</t>
+        </is>
+      </c>
+      <c r="J195" t="inlineStr">
+        <is>
+          <t>관리국의 일부 수감자가 자발적으로 단막극 팀을 만들었다. 현재 함께 반전과 갈등으로 가득한 이야기를 만들어 나갈 각본 작성이 특기인 수감자를 모집하는 중이다.</t>
+        </is>
+      </c>
+      <c r="K195" t="inlineStr">
+        <is>
+          <t>管理局内部分禁闭者自发组建短剧剧组，现决定招募擅长编写的禁闭者加入，协助打造情节跌宕起伏、矛盾火花四溅的剧情。</t>
+        </is>
+      </c>
+      <c r="L195" t="inlineStr">
+        <is>
+          <t>管理局內部分禁閉者自發組建短劇劇組，現決定招募擅長編寫的禁閉者加入，協助打造情節跌宕起伏、矛盾火花四濺的劇情。</t>
+        </is>
+      </c>
+      <c r="M195" t="inlineStr">
+        <is>
+          <t>Irrheia</t>
+        </is>
+      </c>
+      <c r="N195" t="inlineStr">
+        <is>
+          <t>イレイア</t>
+        </is>
+      </c>
+      <c r="O195" t="inlineStr">
+        <is>
+          <t>이레이아</t>
+        </is>
+      </c>
+      <c r="P195" t="inlineStr">
+        <is>
+          <t>伊蕾娅</t>
+        </is>
+      </c>
+      <c r="Q195" t="inlineStr">
+        <is>
+          <t>伊蕾婭</t>
+        </is>
+      </c>
+      <c r="R195" t="inlineStr"/>
+      <c r="S195" t="inlineStr"/>
+      <c r="T195" t="inlineStr"/>
+      <c r="U195" t="inlineStr"/>
+      <c r="V195" t="inlineStr"/>
+      <c r="W195" t="inlineStr">
+        <is>
+          <t>DisCoins</t>
+        </is>
+      </c>
+      <c r="X195" t="inlineStr">
+        <is>
+          <t>ディスコイン</t>
+        </is>
+      </c>
+      <c r="Y195" t="inlineStr">
+        <is>
+          <t>디스코인</t>
+        </is>
+      </c>
+      <c r="Z195" t="inlineStr">
+        <is>
+          <t>狄斯币</t>
+        </is>
+      </c>
+      <c r="AA195" t="inlineStr">
+        <is>
+          <t>狄斯幣</t>
+        </is>
+      </c>
+      <c r="AB195" t="inlineStr">
+        <is>
+          <t>8000.0</t>
+        </is>
+      </c>
+      <c r="AC195" t="inlineStr">
+        <is>
+          <t>DisCoins</t>
+        </is>
+      </c>
+      <c r="AD195" t="inlineStr">
+        <is>
+          <t>ディスコイン</t>
+        </is>
+      </c>
+      <c r="AE195" t="inlineStr">
+        <is>
+          <t>디스코인</t>
+        </is>
+      </c>
+      <c r="AF195" t="inlineStr">
+        <is>
+          <t>狄斯币</t>
+        </is>
+      </c>
+      <c r="AG195" t="inlineStr">
+        <is>
+          <t>狄斯幣</t>
+        </is>
+      </c>
+      <c r="AH195" t="inlineStr">
+        <is>
+          <t>2000.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="n">
+        <v>1061002</v>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>Green</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>Illumination Needed</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>照明支援</t>
+        </is>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>조명 지원</t>
+        </is>
+      </c>
+      <c r="F196" t="inlineStr">
+        <is>
+          <t>照明支援</t>
+        </is>
+      </c>
+      <c r="G196" t="inlineStr">
+        <is>
+          <t>照明支援</t>
+        </is>
+      </c>
+      <c r="H196" t="inlineStr">
+        <is>
+          <t>Gang conflicts in Syndicate have caused a partial blackout, leaving residents in a crisis. The Public Security Bureau has issued an emergency notice requesting the Bureau to send Sinners to provide illumination and humanitarian aid.</t>
+        </is>
+      </c>
+      <c r="I196" t="inlineStr">
+        <is>
+          <t>シンジケートエリアでマフィアの抗争により局所的な停電が発生し、現地住民が窮地に陥っている。治安局は緊急通達を出し、必要な照明と生活支援を提供するため、管理局にコンビクトの派遣を要請した。</t>
+        </is>
+      </c>
+      <c r="J196" t="inlineStr">
+        <is>
+          <t>신디케이트 구역에서 갱단 간의 충돌로 인해 일부 구역에 정전이 일어나 현지인들이 곤경에 처했다. 이에 치안국은 긴급 공지를 발표해, 관리국에서 수감자를 파견해 필수적인 조명과 생활 물자 지원을 수행해 줄 것을 요청했다.</t>
+        </is>
+      </c>
+      <c r="K196" t="inlineStr">
+        <is>
+          <t>辛迪加区域因帮派冲突引发局部停电，当地民众陷入困境。治安局发出紧急通告，请求管理局派遣禁闭者前往，提供必要的照明与生活支援。</t>
+        </is>
+      </c>
+      <c r="L196" t="inlineStr">
+        <is>
+          <t>辛迪加區域因幫派衝突引發局部停電，當地民眾陷入困境。治安局發出緊急通告，請求管理局派遣禁閉者前往，提供必要的照明與生活支援。</t>
+        </is>
+      </c>
+      <c r="M196" t="inlineStr">
+        <is>
+          <t>Rumina</t>
+        </is>
+      </c>
+      <c r="N196" t="inlineStr">
+        <is>
+          <t>ルミナ</t>
+        </is>
+      </c>
+      <c r="O196" t="inlineStr">
+        <is>
+          <t>루미나</t>
+        </is>
+      </c>
+      <c r="P196" t="inlineStr">
+        <is>
+          <t>露米娜</t>
+        </is>
+      </c>
+      <c r="Q196" t="inlineStr">
+        <is>
+          <t>露米娜</t>
+        </is>
+      </c>
+      <c r="R196" t="inlineStr"/>
+      <c r="S196" t="inlineStr"/>
+      <c r="T196" t="inlineStr"/>
+      <c r="U196" t="inlineStr"/>
+      <c r="V196" t="inlineStr"/>
+      <c r="W196" t="inlineStr">
+        <is>
+          <t>Hypercube</t>
+        </is>
+      </c>
+      <c r="X196" t="inlineStr">
+        <is>
+          <t>イレギュラーキューブ</t>
+        </is>
+      </c>
+      <c r="Y196" t="inlineStr">
+        <is>
+          <t>큐브</t>
+        </is>
+      </c>
+      <c r="Z196" t="inlineStr">
+        <is>
+          <t>异方晶</t>
+        </is>
+      </c>
+      <c r="AA196" t="inlineStr">
+        <is>
+          <t>異方晶</t>
+        </is>
+      </c>
+      <c r="AB196" t="inlineStr">
+        <is>
+          <t>10.0</t>
+        </is>
+      </c>
+      <c r="AC196" t="inlineStr">
+        <is>
+          <t>Hypercube</t>
+        </is>
+      </c>
+      <c r="AD196" t="inlineStr">
+        <is>
+          <t>イレギュラーキューブ</t>
+        </is>
+      </c>
+      <c r="AE196" t="inlineStr">
+        <is>
+          <t>큐브</t>
+        </is>
+      </c>
+      <c r="AF196" t="inlineStr">
+        <is>
+          <t>异方晶</t>
+        </is>
+      </c>
+      <c r="AG196" t="inlineStr">
+        <is>
+          <t>異方晶</t>
+        </is>
+      </c>
+      <c r="AH196" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="n">
+        <v>1061003</v>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>Blue</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>Safety Seminar</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>安全講座</t>
+        </is>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>안전 교육</t>
+        </is>
+      </c>
+      <c r="F197" t="inlineStr">
+        <is>
+          <t>安全讲座</t>
+        </is>
+      </c>
+      <c r="G197" t="inlineStr">
+        <is>
+          <t>安全講座</t>
+        </is>
+      </c>
+      <c r="H197" t="inlineStr">
+        <is>
+          <t>The Public Security Bureau will be hosting a household fire safety seminar to raise public safety awareness. Certain Sinners within the Bureau are required to attend and will now be selected together.</t>
+        </is>
+      </c>
+      <c r="I197" t="inlineStr">
+        <is>
+          <t>治安局は一般市民の防災意識向上のため、住宅火災の安全教育講座を開催することにした。管理局内の一部コンビクトも参加必須名簿に記載されており、人員を一斉に現地へ向かわせる必要がある。</t>
+        </is>
+      </c>
+      <c r="J197" t="inlineStr">
+        <is>
+          <t>시민들의 안전 의식을 높이기 위해 치안국은 가정 내 화재 안전 교육을 진행할 예정이다. 관리국의 일부 수감자가 의무 참석 대상자로 지정되었으며, 인원을 일괄적으로 편성해 현장에 파견해야 한다.</t>
+        </is>
+      </c>
+      <c r="K197" t="inlineStr">
+        <is>
+          <t>治安局将举办家庭用火安全教育讲座，旨在提升公众防护意识。管理局内部分禁闭者被列入必须参加的名单，现统一安排人员前往。</t>
+        </is>
+      </c>
+      <c r="L197" t="inlineStr">
+        <is>
+          <t>治安局將舉辦家庭用火安全教育講座，旨在提升公眾防護意識。管理局內部分禁閉者被列入必須參加的名單，現統一安排人員前往。</t>
+        </is>
+      </c>
+      <c r="M197" t="inlineStr">
+        <is>
+          <t>Rumina</t>
+        </is>
+      </c>
+      <c r="N197" t="inlineStr">
+        <is>
+          <t>ルミナ</t>
+        </is>
+      </c>
+      <c r="O197" t="inlineStr">
+        <is>
+          <t>루미나</t>
+        </is>
+      </c>
+      <c r="P197" t="inlineStr">
+        <is>
+          <t>露米娜</t>
+        </is>
+      </c>
+      <c r="Q197" t="inlineStr">
+        <is>
+          <t>露米娜</t>
+        </is>
+      </c>
+      <c r="R197" t="inlineStr">
+        <is>
+          <t>Flora</t>
+        </is>
+      </c>
+      <c r="S197" t="inlineStr">
+        <is>
+          <t>フローラ</t>
+        </is>
+      </c>
+      <c r="T197" t="inlineStr">
+        <is>
+          <t>플로라</t>
+        </is>
+      </c>
+      <c r="U197" t="inlineStr">
+        <is>
+          <t>芙洛拉</t>
+        </is>
+      </c>
+      <c r="V197" t="inlineStr">
+        <is>
+          <t>芙洛拉</t>
+        </is>
+      </c>
+      <c r="W197" t="inlineStr">
+        <is>
+          <t>Mania Essence</t>
+        </is>
+      </c>
+      <c r="X197" t="inlineStr">
+        <is>
+          <t>ルナティックエッセンス</t>
+        </is>
+      </c>
+      <c r="Y197" t="inlineStr">
+        <is>
+          <t>광란의 정수</t>
+        </is>
+      </c>
+      <c r="Z197" t="inlineStr">
+        <is>
+          <t>狂乱精粹</t>
+        </is>
+      </c>
+      <c r="AA197" t="inlineStr">
+        <is>
+          <t>狂亂精粹</t>
+        </is>
+      </c>
+      <c r="AB197" t="inlineStr">
+        <is>
+          <t>4000.0</t>
+        </is>
+      </c>
+      <c r="AC197" t="inlineStr">
+        <is>
+          <t>Mania Essence</t>
+        </is>
+      </c>
+      <c r="AD197" t="inlineStr">
+        <is>
+          <t>ルナティックエッセンス</t>
+        </is>
+      </c>
+      <c r="AE197" t="inlineStr">
+        <is>
+          <t>광란의 정수</t>
+        </is>
+      </c>
+      <c r="AF197" t="inlineStr">
+        <is>
+          <t>狂乱精粹</t>
+        </is>
+      </c>
+      <c r="AG197" t="inlineStr">
+        <is>
+          <t>狂亂精粹</t>
+        </is>
+      </c>
+      <c r="AH197" t="inlineStr">
+        <is>
+          <t>1000.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="n">
+        <v>1062001</v>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>Purple</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>Charity Ambassador</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>チャリティー大使</t>
+        </is>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>자선가</t>
+        </is>
+      </c>
+      <c r="F198" t="inlineStr">
+        <is>
+          <t>慈善大使</t>
+        </is>
+      </c>
+      <c r="G198" t="inlineStr">
+        <is>
+          <t>慈善大使</t>
+        </is>
+      </c>
+      <c r="H198" t="inlineStr">
+        <is>
+          <t>Reports indicate that an alleged Mania-contaminated item has appeared at a private charity auction in Eastside. A reputable figure in philanthropic circles is urgently needed to serve as an intermediary, facilitating the Bureau's investigation into the item.</t>
+        </is>
+      </c>
+      <c r="I198" t="inlineStr">
+        <is>
+          <t>ニューシティで行われる非公開のチャリティーオークションに、狂瞳汚染の疑いがある品が出品されているとの情報が入った。管理局が品物の調査をしやすくするため、慈善事業で高い評価のある人物による仲立ちが急ぎ求められている。</t>
+        </is>
+      </c>
+      <c r="J198" t="inlineStr">
+        <is>
+          <t>소식에 따르면, 신성에서 비밀리에 진행된 한 자선 경매에 변이 오염을 지닌 경매품이 등장했다고 한다. 관리국이 해당 경매품을 조사할 수 있도록 자선 분야에서 명망이 높은 인물이 알선 역할을 맡아야 한다.</t>
+        </is>
+      </c>
+      <c r="K198" t="inlineStr">
+        <is>
+          <t>有消息称，新城一场不对外公开的慈善拍卖上疑似出现携带狂厄污染的拍品，急需一位在慈善事业上颇有名望的人员从中斡旋牵线，方便管理局介入拍品的调查。</t>
+        </is>
+      </c>
+      <c r="L198" t="inlineStr">
+        <is>
+          <t>有消息稱，新城一場不對外公開的慈善拍賣上疑似出現攜帶狂厄汙染的拍賣品，急需一位在慈善事業上頗有名望的人員從中斡旋牽線，方便管理局介入拍賣品的調查。</t>
+        </is>
+      </c>
+      <c r="M198" t="inlineStr">
+        <is>
+          <t>Margaret</t>
+        </is>
+      </c>
+      <c r="N198" t="inlineStr">
+        <is>
+          <t>マルガリータ</t>
+        </is>
+      </c>
+      <c r="O198" t="inlineStr">
+        <is>
+          <t>마가렛</t>
+        </is>
+      </c>
+      <c r="P198" t="inlineStr">
+        <is>
+          <t>玛格丽塔</t>
+        </is>
+      </c>
+      <c r="Q198" t="inlineStr">
+        <is>
+          <t>瑪格麗塔</t>
+        </is>
+      </c>
+      <c r="R198" t="inlineStr"/>
+      <c r="S198" t="inlineStr"/>
+      <c r="T198" t="inlineStr"/>
+      <c r="U198" t="inlineStr"/>
+      <c r="V198" t="inlineStr"/>
+      <c r="W198" t="inlineStr">
+        <is>
+          <t>DisCoins</t>
+        </is>
+      </c>
+      <c r="X198" t="inlineStr">
+        <is>
+          <t>ディスコイン</t>
+        </is>
+      </c>
+      <c r="Y198" t="inlineStr">
+        <is>
+          <t>디스코인</t>
+        </is>
+      </c>
+      <c r="Z198" t="inlineStr">
+        <is>
+          <t>狄斯币</t>
+        </is>
+      </c>
+      <c r="AA198" t="inlineStr">
+        <is>
+          <t>狄斯幣</t>
+        </is>
+      </c>
+      <c r="AB198" t="inlineStr">
+        <is>
+          <t>8000.0</t>
+        </is>
+      </c>
+      <c r="AC198" t="inlineStr">
+        <is>
+          <t>DisCoins</t>
+        </is>
+      </c>
+      <c r="AD198" t="inlineStr">
+        <is>
+          <t>ディスコイン</t>
+        </is>
+      </c>
+      <c r="AE198" t="inlineStr">
+        <is>
+          <t>디스코인</t>
+        </is>
+      </c>
+      <c r="AF198" t="inlineStr">
+        <is>
+          <t>狄斯币</t>
+        </is>
+      </c>
+      <c r="AG198" t="inlineStr">
+        <is>
+          <t>狄斯幣</t>
+        </is>
+      </c>
+      <c r="AH198" t="inlineStr">
+        <is>
+          <t>2000.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="n">
+        <v>1062002</v>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>Purple</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>Dangerous Research</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>危険な研究</t>
+        </is>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>위험한 연구</t>
+        </is>
+      </c>
+      <c r="F199" t="inlineStr">
+        <is>
+          <t>危险研究</t>
+        </is>
+      </c>
+      <c r="G199" t="inlineStr">
+        <is>
+          <t>危險研究</t>
+        </is>
+      </c>
+      <c r="H199" t="inlineStr">
+        <is>
+          <t>The Ring Research Institute is sending an academic team to conduct observations and surveys near a Black Ring ruin. A Sinner who is knowledgeable about the interior structure of a Black Ring is required to accompany the team and ensure the researchers' safety.</t>
+        </is>
+      </c>
+      <c r="I199" t="inlineStr">
+        <is>
+          <t>リング研究所が、ブラックリング遺跡周辺で観測と調査を行う学術チームを派遣することになった。それにあたり、研究員の安全を確保するため、ブラックリング内部に詳しいコンビクトの同行が必要とされている。</t>
+        </is>
+      </c>
+      <c r="J199" t="inlineStr">
+        <is>
+          <t>링 연구소가 관측 및 조사 작업을 위해 블랙링 유적 인근에 학술 단체를 파견했다. 연구 인원의 안전을 보장하기 위해 블랙링 내부에 대해 이해가 깊은 수감자의 동행이 필요하다.</t>
+        </is>
+      </c>
+      <c r="K199" t="inlineStr">
+        <is>
+          <t>环研究院派出学术团体在黑环遗迹附近进行观测与考察，需要一位对黑环内部了解较为深入的禁闭者陪同，以保证科研人员的人身安全。</t>
+        </is>
+      </c>
+      <c r="L199" t="inlineStr">
+        <is>
+          <t>環研究院派出學術團體在黑環遺跡附近進行觀測與考察，需要一位對黑環內部瞭解較為深入的禁閉者陪同，以確保研究人員的人身安全。</t>
+        </is>
+      </c>
+      <c r="M199" t="inlineStr">
+        <is>
+          <t>Rust</t>
+        </is>
+      </c>
+      <c r="N199" t="inlineStr">
+        <is>
+          <t>錆</t>
+        </is>
+      </c>
+      <c r="O199" t="inlineStr">
+        <is>
+          <t>러스트</t>
+        </is>
+      </c>
+      <c r="P199" t="inlineStr">
+        <is>
+          <t>锈</t>
+        </is>
+      </c>
+      <c r="Q199" t="inlineStr">
+        <is>
+          <t>鏽</t>
+        </is>
+      </c>
+      <c r="R199" t="inlineStr"/>
+      <c r="S199" t="inlineStr"/>
+      <c r="T199" t="inlineStr"/>
+      <c r="U199" t="inlineStr"/>
+      <c r="V199" t="inlineStr"/>
+      <c r="W199" t="inlineStr">
+        <is>
+          <t>Red Crystal</t>
+        </is>
+      </c>
+      <c r="X199" t="inlineStr">
+        <is>
+          <t>赤の結晶</t>
+        </is>
+      </c>
+      <c r="Y199" t="inlineStr">
+        <is>
+          <t>붉은 결정</t>
+        </is>
+      </c>
+      <c r="Z199" t="inlineStr">
+        <is>
+          <t>赤晶</t>
+        </is>
+      </c>
+      <c r="AA199" t="inlineStr">
+        <is>
+          <t>赤晶</t>
+        </is>
+      </c>
+      <c r="AB199" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AC199" t="inlineStr">
+        <is>
+          <t>Red Stone Concentrate</t>
+        </is>
+      </c>
+      <c r="AD199" t="inlineStr">
+        <is>
+          <t>赤石の精鉱</t>
+        </is>
+      </c>
+      <c r="AE199" t="inlineStr">
+        <is>
+          <t>정교한 레드 스톤 광석</t>
+        </is>
+      </c>
+      <c r="AF199" t="inlineStr">
+        <is>
+          <t>红石精矿</t>
+        </is>
+      </c>
+      <c r="AG199" t="inlineStr">
+        <is>
+          <t>紅石精礦</t>
+        </is>
+      </c>
+      <c r="AH199" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="n">
+        <v>1062003</v>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>Green</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>Reticle Sniper</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>精密狙撃</t>
+        </is>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>정확한 저격</t>
+        </is>
+      </c>
+      <c r="F200" t="inlineStr">
+        <is>
+          <t>精准狙击</t>
+        </is>
+      </c>
+      <c r="G200" t="inlineStr">
+        <is>
+          <t>精準狙擊</t>
+        </is>
+      </c>
+      <c r="H200" t="inlineStr">
+        <is>
+          <t>A kidnapping case has arisen in a commercial district in Eastside. The kidnapper is highly dangerous, prompting the Public Security Bureau to urgently request a sniper. Requirements: The operative must be capable of engaging from extreme range and neutralizing the target with a single lethal shot.</t>
+        </is>
+      </c>
+      <c r="I200" t="inlineStr">
+        <is>
+          <t>ニューシティの繁華街で人質誘拐事件が発生した。犯人は極めて危険性が高く、治安局は緊急で狙撃手を招集している。条件：超遠距離から射撃し、標的を一撃で仕留めること。</t>
+        </is>
+      </c>
+      <c r="J200" t="inlineStr">
+        <is>
+          <t>신성 번화가에서 인질 납치 사건이 발생했다. 범인의 위험도가 높아 치안국은 긴급히 저격수 한 명을 소집했다. 극한 거리에서 사격할 수 있고 목표를 단 한 발로 사살할 수 있는 정확성을 겸비한 수감자를 파견해야 한다.</t>
+        </is>
+      </c>
+      <c r="K200" t="inlineStr">
+        <is>
+          <t>新城闹市区发生一桩人质绑架案，绑匪危险性较高，治安局特此紧急征召一名狙击手。要求：该人员需要在极限距离下射击，并对目标一击毙命。</t>
+        </is>
+      </c>
+      <c r="L200" t="inlineStr">
+        <is>
+          <t>新城鬧區發生一樁人質綁架案，綁匪危險性較高，治安局特此緊急徵召一名狙擊手。要求：該人員需要在極限距離下射擊，並對目標一擊斃命。</t>
+        </is>
+      </c>
+      <c r="M200" t="inlineStr">
+        <is>
+          <t>Helga</t>
+        </is>
+      </c>
+      <c r="N200" t="inlineStr">
+        <is>
+          <t>ヘルガ</t>
+        </is>
+      </c>
+      <c r="O200" t="inlineStr">
+        <is>
+          <t>헬가</t>
+        </is>
+      </c>
+      <c r="P200" t="inlineStr">
+        <is>
+          <t>荷尔加</t>
+        </is>
+      </c>
+      <c r="Q200" t="inlineStr">
+        <is>
+          <t>荷爾加</t>
+        </is>
+      </c>
+      <c r="R200" t="inlineStr"/>
+      <c r="S200" t="inlineStr"/>
+      <c r="T200" t="inlineStr"/>
+      <c r="U200" t="inlineStr"/>
+      <c r="V200" t="inlineStr"/>
+      <c r="W200" t="inlineStr">
+        <is>
+          <t>Tear Stone Concentrate</t>
+        </is>
+      </c>
+      <c r="X200" t="inlineStr">
+        <is>
+          <t>涙石の精鉱</t>
+        </is>
+      </c>
+      <c r="Y200" t="inlineStr">
+        <is>
+          <t>정교한 눈물석 광석</t>
+        </is>
+      </c>
+      <c r="Z200" t="inlineStr">
+        <is>
+          <t>泪石精矿</t>
+        </is>
+      </c>
+      <c r="AA200" t="inlineStr">
+        <is>
+          <t>淚石精礦</t>
+        </is>
+      </c>
+      <c r="AB200" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AC200" t="inlineStr">
+        <is>
+          <t>Tear Stone Raw Ore</t>
+        </is>
+      </c>
+      <c r="AD200" t="inlineStr">
+        <is>
+          <t>涙石の原鉱</t>
+        </is>
+      </c>
+      <c r="AE200" t="inlineStr">
+        <is>
+          <t>거친 눈물석 광석</t>
+        </is>
+      </c>
+      <c r="AF200" t="inlineStr">
+        <is>
+          <t>泪石粗矿</t>
+        </is>
+      </c>
+      <c r="AG200" t="inlineStr">
+        <is>
+          <t>淚石粗礦</t>
+        </is>
+      </c>
+      <c r="AH200" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="n">
+        <v>1062004</v>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>Blue</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>Killer Drone</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>デスドローン</t>
+        </is>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>죽음의 드론</t>
+        </is>
+      </c>
+      <c r="F201" t="inlineStr">
+        <is>
+          <t>夺命无人机</t>
+        </is>
+      </c>
+      <c r="G201" t="inlineStr">
+        <is>
+          <t>奪命無人機</t>
+        </is>
+      </c>
+      <c r="H201" t="inlineStr">
+        <is>
+          <t>A central system malfunction has occurred at a drone delivery hub in Eastside, causing numerous drones to go haywire over the city and posing a significant public safety hazard. Two Sinners with expertise in machines need to be sent to provide emergency support.</t>
+        </is>
+      </c>
+      <c r="I201" t="inlineStr">
+        <is>
+          <t>ニューシティのあるドローン配送ステーションで中枢機械が故障し、多数のドローンが都市上空で制御不能となっている。安全上のリスクが極めて高いため、機械に精通したコンビクトを2名支援に派遣することになった。</t>
+        </is>
+      </c>
+      <c r="J201" t="inlineStr">
+        <is>
+          <t>신성의 한 드론 배송 거점에서 핵심 기계 고장이 발생해 다수의 드론이 통제 불능 상태에 빠졌다. 안전상 위험이 매우 커, 기계 지식에 능통한 수감자 2명을 특별 파견하여 지원해야 한다.</t>
+        </is>
+      </c>
+      <c r="K201" t="inlineStr">
+        <is>
+          <t>新城某无人机快递配送站点发生中枢机械故障，大量无人机在城市上空失控，安全隐患极大，特此派遣两名精通机械知识的禁闭者前来支援。</t>
+        </is>
+      </c>
+      <c r="L201" t="inlineStr">
+        <is>
+          <t>新城某無人機快遞配送網站發生中樞機械故障，大量無人機在城市上空失控，安全隱患極大，特此派遣兩名精通機械知識的禁閉者前來支援。</t>
+        </is>
+      </c>
+      <c r="M201" t="inlineStr">
+        <is>
+          <t>Helga</t>
+        </is>
+      </c>
+      <c r="N201" t="inlineStr">
+        <is>
+          <t>ヘルガ</t>
+        </is>
+      </c>
+      <c r="O201" t="inlineStr">
+        <is>
+          <t>헬가</t>
+        </is>
+      </c>
+      <c r="P201" t="inlineStr">
+        <is>
+          <t>荷尔加</t>
+        </is>
+      </c>
+      <c r="Q201" t="inlineStr">
+        <is>
+          <t>荷爾加</t>
+        </is>
+      </c>
+      <c r="R201" t="inlineStr">
+        <is>
+          <t>Eureka</t>
+        </is>
+      </c>
+      <c r="S201" t="inlineStr">
+        <is>
+          <t>エウレカ</t>
+        </is>
+      </c>
+      <c r="T201" t="inlineStr">
+        <is>
+          <t>유레카</t>
+        </is>
+      </c>
+      <c r="U201" t="inlineStr">
+        <is>
+          <t>优利卡</t>
+        </is>
+      </c>
+      <c r="V201" t="inlineStr">
+        <is>
+          <t>優利卡</t>
+        </is>
+      </c>
+      <c r="W201" t="inlineStr">
+        <is>
+          <t>Bronze Concentrate</t>
+        </is>
+      </c>
+      <c r="X201" t="inlineStr">
+        <is>
+          <t>曲銅の精鉱</t>
+        </is>
+      </c>
+      <c r="Y201" t="inlineStr">
+        <is>
+          <t>정교한 곡선형 구리 광석</t>
+        </is>
+      </c>
+      <c r="Z201" t="inlineStr">
+        <is>
+          <t>曲铜精矿</t>
+        </is>
+      </c>
+      <c r="AA201" t="inlineStr">
+        <is>
+          <t>曲銅精礦</t>
+        </is>
+      </c>
+      <c r="AB201" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AC201" t="inlineStr">
+        <is>
+          <t>Bronze Concentrate</t>
+        </is>
+      </c>
+      <c r="AD201" t="inlineStr">
+        <is>
+          <t>曲銅の精鉱</t>
+        </is>
+      </c>
+      <c r="AE201" t="inlineStr">
+        <is>
+          <t>정교한 곡선형 구리 광석</t>
+        </is>
+      </c>
+      <c r="AF201" t="inlineStr">
+        <is>
+          <t>曲铜精矿</t>
+        </is>
+      </c>
+      <c r="AG201" t="inlineStr">
+        <is>
+          <t>曲銅精礦</t>
+        </is>
+      </c>
+      <c r="AH201" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="n">
+        <v>1063001</v>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>Purple</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>Mysticism Fraud Busting</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>玄学詐欺の摘発</t>
+        </is>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>현학 사기</t>
+        </is>
+      </c>
+      <c r="F202" t="inlineStr">
+        <is>
+          <t>玄学打假</t>
+        </is>
+      </c>
+      <c r="G202" t="inlineStr">
+        <is>
+          <t>玄學打假</t>
+        </is>
+      </c>
+      <c r="H202" t="inlineStr">
+        <is>
+          <t>Recently, a fraud ring has emerged in Eastside, using Eastian mysticism as a front for their scams. Due to their sophisticated methods, many citizens have been swindled and lost everything. The Bureau has been requested to send an expert well-versed in Eastian folklore to assist in solving this case.</t>
+        </is>
+      </c>
+      <c r="I202" t="inlineStr">
+        <is>
+          <t>最近、ニューシティで東洲の玄学を騙り詐欺を働くグループが現れた。その巧妙な手口により多数の市民が被害に遭い、全財産を失う事態となっている。よって管理局に対し、東洲の民俗に精通した専門家を派遣し、事件解決に協力するよう申請する。</t>
+        </is>
+      </c>
+      <c r="J202" t="inlineStr">
+        <is>
+          <t>최근 신성에 동방 대륙의 현학을 내세워 사기를 치는 무리가 출몰했고, 이들의 사기 수법이 치밀해 많은 피해자가 재산을 잃었다. 현재 관리국은 동방 대륙 민속에 대해 잘 아는 전문가를 파견하여 수사를 지원해야 한다.</t>
+        </is>
+      </c>
+      <c r="K202" t="inlineStr">
+        <is>
+          <t>近日，新城出现一伙以东洲玄学为旗号招摇撞骗的诈骗团伙，因其骗术高超，致多名市民受骗血本无归。现特向管理局申请派遣一位精通东洲民俗的专家前往协助破案。</t>
+        </is>
+      </c>
+      <c r="L202" t="inlineStr">
+        <is>
+          <t>近日，新城出現一夥以東洲玄學為旗號招搖撞騙的詐騙集團，因其騙術高超，致多名市民受騙血本無歸。現特向管理局申請派遣一位精通東洲民俗的專家前往協助破案。</t>
+        </is>
+      </c>
+      <c r="M202" t="inlineStr">
+        <is>
+          <t>Lichen</t>
+        </is>
+      </c>
+      <c r="N202" t="inlineStr">
+        <is>
+          <t>離塵</t>
+        </is>
+      </c>
+      <c r="O202" t="inlineStr">
+        <is>
+          <t>리진</t>
+        </is>
+      </c>
+      <c r="P202" t="inlineStr">
+        <is>
+          <t>离尘</t>
+        </is>
+      </c>
+      <c r="Q202" t="inlineStr">
+        <is>
+          <t>離塵</t>
+        </is>
+      </c>
+      <c r="R202" t="inlineStr"/>
+      <c r="S202" t="inlineStr"/>
+      <c r="T202" t="inlineStr"/>
+      <c r="U202" t="inlineStr"/>
+      <c r="V202" t="inlineStr"/>
+      <c r="W202" t="inlineStr">
+        <is>
+          <t>Infected Tentacle</t>
+        </is>
+      </c>
+      <c r="X202" t="inlineStr">
+        <is>
+          <t>感染された触手</t>
+        </is>
+      </c>
+      <c r="Y202" t="inlineStr">
+        <is>
+          <t>감염된 다리</t>
+        </is>
+      </c>
+      <c r="Z202" t="inlineStr">
+        <is>
+          <t>感染腕足</t>
+        </is>
+      </c>
+      <c r="AA202" t="inlineStr">
+        <is>
+          <t>感染腕足</t>
+        </is>
+      </c>
+      <c r="AB202" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AC202" t="inlineStr">
+        <is>
+          <t>Organic Tentacle</t>
+        </is>
+      </c>
+      <c r="AD202" t="inlineStr">
+        <is>
+          <t>原生触手</t>
+        </is>
+      </c>
+      <c r="AE202" t="inlineStr">
+        <is>
+          <t>원시적 다리</t>
+        </is>
+      </c>
+      <c r="AF202" t="inlineStr">
+        <is>
+          <t>原生腕足</t>
+        </is>
+      </c>
+      <c r="AG202" t="inlineStr">
+        <is>
+          <t>原生腕足</t>
+        </is>
+      </c>
+      <c r="AH202" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="n">
+        <v>1099001</v>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>Green</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>Dream Interpretation</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>夢の解析</t>
+        </is>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>꿈의 해석</t>
+        </is>
+      </c>
+      <c r="F203" t="inlineStr">
+        <is>
+          <t>梦的解析</t>
+        </is>
+      </c>
+      <c r="G203" t="inlineStr">
+        <is>
+          <t>夢的解析</t>
+        </is>
+      </c>
+      <c r="H203" t="inlineStr">
+        <is>
+          <t>Residents in some areas of Eastside often suffer from nightmares. It is necessary to find out why.</t>
+        </is>
+      </c>
+      <c r="I203" t="inlineStr">
+        <is>
+          <t>ニューシティの一部エリアの住民がよくナイトメアにうなされている。具体的な原因を調査しなければならない。</t>
+        </is>
+      </c>
+      <c r="J203" t="inlineStr">
+        <is>
+          <t>신성 일부 지역 주민들은 악몽을 자주꾼다. 구체적인 원인을 철저히 조사해야 한다.</t>
+        </is>
+      </c>
+      <c r="K203" t="inlineStr">
+        <is>
+          <t>新城一些区域的居民经常做噩梦，需要查清具体原因。</t>
+        </is>
+      </c>
+      <c r="L203" t="inlineStr">
+        <is>
+          <t>新城一些區域的居民經常做惡夢，需要查明具體原因。</t>
+        </is>
+      </c>
+      <c r="M203" t="inlineStr">
+        <is>
+          <t>Hecate</t>
+        </is>
+      </c>
+      <c r="N203" t="inlineStr">
+        <is>
+          <t>ヘカテー</t>
+        </is>
+      </c>
+      <c r="O203" t="inlineStr">
+        <is>
+          <t>헤카테</t>
+        </is>
+      </c>
+      <c r="P203" t="inlineStr">
+        <is>
+          <t>赫卡蒂</t>
+        </is>
+      </c>
+      <c r="Q203" t="inlineStr">
+        <is>
+          <t>赫卡蒂</t>
+        </is>
+      </c>
+      <c r="R203" t="inlineStr"/>
+      <c r="S203" t="inlineStr"/>
+      <c r="T203" t="inlineStr"/>
+      <c r="U203" t="inlineStr"/>
+      <c r="V203" t="inlineStr"/>
+      <c r="W203" t="inlineStr">
+        <is>
           <t>Arsenopyrite Concentrate</t>
         </is>
       </c>
-      <c r="X194" t="inlineStr">
+      <c r="X203" t="inlineStr">
         <is>
           <t>毒砂の精鉱</t>
         </is>
       </c>
-      <c r="Y194" t="inlineStr">
+      <c r="Y203" t="inlineStr">
         <is>
           <t>정교한 독모래 광석</t>
         </is>
       </c>
-      <c r="Z194" t="inlineStr">
+      <c r="Z203" t="inlineStr">
         <is>
           <t>毒砂精矿</t>
         </is>
       </c>
-      <c r="AA194" t="inlineStr">
+      <c r="AA203" t="inlineStr">
         <is>
           <t>毒砂精礦</t>
         </is>
       </c>
-      <c r="AB194" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="AC194" t="inlineStr">
+      <c r="AB203" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AC203" t="inlineStr">
         <is>
           <t>Arsenopyrite Raw Ore</t>
         </is>
       </c>
-      <c r="AD194" t="inlineStr">
+      <c r="AD203" t="inlineStr">
         <is>
           <t>毒砂の原鉱</t>
         </is>
       </c>
-      <c r="AE194" t="inlineStr">
+      <c r="AE203" t="inlineStr">
         <is>
           <t>거친 독모래 광석</t>
         </is>
       </c>
-      <c r="AF194" t="inlineStr">
+      <c r="AF203" t="inlineStr">
         <is>
           <t>毒砂粗矿</t>
         </is>
       </c>
-      <c r="AG194" t="inlineStr">
+      <c r="AG203" t="inlineStr">
         <is>
           <t>毒砂粗礦</t>
         </is>
       </c>
-      <c r="AH194" t="inlineStr">
+      <c r="AH203" t="inlineStr">
         <is>
           <t>1.0</t>
         </is>

</xml_diff>